<commit_message>
Atualiza planilha custos Olaria
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/CUSTOS OLARIA.xlsx
+++ b/data/CUSTOS OLARIA.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\CONTROLE DE DESPESAS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lélisson\Desktop\RELATORIOS  AUTOMATICOS\controle de gastos galpoes\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{776E08AD-4B66-4D8F-8A82-C8675AD9AEEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="15345" windowHeight="4185" tabRatio="500"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DASHBOARD" sheetId="1" r:id="rId1"/>
@@ -22,7 +23,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="0">DASHBOARD!$A$1:$AA$69</definedName>
     <definedName name="Periodo">DASHBOARD!$U$3</definedName>
   </definedNames>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -44,12 +45,12 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Unknown Author</author>
   </authors>
   <commentList>
-    <comment ref="D4" authorId="0" shapeId="0">
+    <comment ref="D4" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0400-000001000000}">
       <text>
         <r>
           <rPr>
@@ -61,7 +62,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F4" authorId="0" shapeId="0">
+    <comment ref="F4" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0400-000002000000}">
       <text>
         <r>
           <rPr>
@@ -422,7 +423,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="7">
     <numFmt numFmtId="44" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="&quot;R$ &quot;#,##0"/>
@@ -1060,41 +1061,59 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="166" fontId="10" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="10" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="168" fontId="8" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="1" fontId="8" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="14" fillId="4" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="14" fillId="4" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="166" fontId="13" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="14" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="13" fillId="4" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="10" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -1132,59 +1151,41 @@
     <xf numFmtId="0" fontId="8" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="13" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="1" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="14" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="13" fillId="4" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="14" fillId="4" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="14" fillId="4" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="10" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="10" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="8" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="8" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="8" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1559,7 +1560,7 @@
                   <c:v>35256.051666666666</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0</c:v>
+                  <c:v>3379.49</c:v>
                 </c:pt>
                 <c:pt idx="9">
                   <c:v>0</c:v>
@@ -2028,7 +2029,6 @@
     </c:plotArea>
     <c:legend>
       <c:legendPos val="t"/>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -2224,7 +2224,6 @@
           <c:dLbls>
             <c:dLbl>
               <c:idx val="0"/>
-              <c:layout/>
               <c:spPr/>
               <c:txPr>
                 <a:bodyPr wrap="square"/>
@@ -2248,9 +2247,7 @@
               <c:showPercent val="1"/>
               <c:showBubbleSize val="1"/>
               <c:extLst>
-                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                  <c15:layout/>
-                </c:ext>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                   <c16:uniqueId val="{00000001-3A68-42A7-B53D-2E82D222E5E4}"/>
                 </c:ext>
@@ -2258,7 +2255,6 @@
             </c:dLbl>
             <c:dLbl>
               <c:idx val="1"/>
-              <c:layout/>
               <c:spPr/>
               <c:txPr>
                 <a:bodyPr wrap="square"/>
@@ -2282,9 +2278,7 @@
               <c:showPercent val="1"/>
               <c:showBubbleSize val="1"/>
               <c:extLst>
-                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                  <c15:layout/>
-                </c:ext>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                   <c16:uniqueId val="{00000003-3A68-42A7-B53D-2E82D222E5E4}"/>
                 </c:ext>
@@ -2292,7 +2286,6 @@
             </c:dLbl>
             <c:dLbl>
               <c:idx val="2"/>
-              <c:layout/>
               <c:spPr/>
               <c:txPr>
                 <a:bodyPr wrap="square"/>
@@ -2316,9 +2309,7 @@
               <c:showPercent val="1"/>
               <c:showBubbleSize val="1"/>
               <c:extLst>
-                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                  <c15:layout/>
-                </c:ext>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                   <c16:uniqueId val="{00000005-3A68-42A7-B53D-2E82D222E5E4}"/>
                 </c:ext>
@@ -2326,7 +2317,6 @@
             </c:dLbl>
             <c:dLbl>
               <c:idx val="3"/>
-              <c:layout/>
               <c:spPr/>
               <c:txPr>
                 <a:bodyPr wrap="square"/>
@@ -2350,9 +2340,7 @@
               <c:showPercent val="1"/>
               <c:showBubbleSize val="1"/>
               <c:extLst>
-                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                  <c15:layout/>
-                </c:ext>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                   <c16:uniqueId val="{00000007-3A68-42A7-B53D-2E82D222E5E4}"/>
                 </c:ext>
@@ -2360,7 +2348,6 @@
             </c:dLbl>
             <c:dLbl>
               <c:idx val="4"/>
-              <c:layout/>
               <c:spPr/>
               <c:txPr>
                 <a:bodyPr wrap="square"/>
@@ -2384,9 +2371,7 @@
               <c:showPercent val="1"/>
               <c:showBubbleSize val="1"/>
               <c:extLst>
-                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                  <c15:layout/>
-                </c:ext>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                   <c16:uniqueId val="{00000009-3A68-42A7-B53D-2E82D222E5E4}"/>
                 </c:ext>
@@ -2693,7 +2678,7 @@
                   <c:v>30733.02</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>27035.919999999991</c:v>
+                  <c:v>30415.409999999989</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>10623</c:v>
@@ -2976,7 +2961,6 @@
     </c:plotArea>
     <c:legend>
       <c:legendPos val="t"/>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -3336,7 +3320,7 @@
                   <c:v>35256.051666666666</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0</c:v>
+                  <c:v>3379.49</c:v>
                 </c:pt>
                 <c:pt idx="9">
                   <c:v>0</c:v>
@@ -4089,57 +4073,57 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <tabColor rgb="FF000000"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:BH69"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="1.5703125" style="1" customWidth="1"/>
-    <col min="2" max="27" width="6.85546875" style="1" customWidth="1"/>
-    <col min="28" max="28" width="1.5703125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="1.5546875" style="1" customWidth="1"/>
+    <col min="2" max="27" width="6.88671875" style="1" customWidth="1"/>
+    <col min="28" max="28" width="1.5546875" style="1" customWidth="1"/>
     <col min="29" max="60" width="13" style="1" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:60" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:60" ht="43.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2"/>
-      <c r="B1" s="56" t="s">
+      <c r="B1" s="91" t="s">
         <v>100</v>
       </c>
-      <c r="C1" s="56"/>
-      <c r="D1" s="56"/>
-      <c r="E1" s="56"/>
-      <c r="F1" s="56"/>
-      <c r="G1" s="56"/>
-      <c r="H1" s="56"/>
-      <c r="I1" s="56"/>
-      <c r="J1" s="56"/>
-      <c r="K1" s="56"/>
-      <c r="L1" s="56"/>
-      <c r="M1" s="56"/>
-      <c r="N1" s="56"/>
-      <c r="O1" s="56"/>
-      <c r="P1" s="56"/>
-      <c r="Q1" s="56"/>
-      <c r="R1" s="56"/>
-      <c r="S1" s="56"/>
-      <c r="T1" s="56"/>
-      <c r="U1" s="56"/>
-      <c r="V1" s="56"/>
-      <c r="W1" s="56"/>
-      <c r="X1" s="56"/>
-      <c r="Y1" s="56"/>
-      <c r="Z1" s="56"/>
-      <c r="AA1" s="56"/>
+      <c r="C1" s="91"/>
+      <c r="D1" s="91"/>
+      <c r="E1" s="91"/>
+      <c r="F1" s="91"/>
+      <c r="G1" s="91"/>
+      <c r="H1" s="91"/>
+      <c r="I1" s="91"/>
+      <c r="J1" s="91"/>
+      <c r="K1" s="91"/>
+      <c r="L1" s="91"/>
+      <c r="M1" s="91"/>
+      <c r="N1" s="91"/>
+      <c r="O1" s="91"/>
+      <c r="P1" s="91"/>
+      <c r="Q1" s="91"/>
+      <c r="R1" s="91"/>
+      <c r="S1" s="91"/>
+      <c r="T1" s="91"/>
+      <c r="U1" s="91"/>
+      <c r="V1" s="91"/>
+      <c r="W1" s="91"/>
+      <c r="X1" s="91"/>
+      <c r="Y1" s="91"/>
+      <c r="Z1" s="91"/>
+      <c r="AA1" s="91"/>
       <c r="AB1" s="4"/>
       <c r="AD1" s="1">
         <f>IF($U$3="Ano",1,MATCH($U$3,Lançamentos!$C$4:$N$4,0))</f>
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:60" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:60" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2"/>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -4169,95 +4153,95 @@
       <c r="AA2" s="3"/>
       <c r="AB2" s="4"/>
     </row>
-    <row r="3" spans="1:60" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:60" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
-      <c r="B3" s="57" t="s">
-        <v>0</v>
-      </c>
-      <c r="C3" s="57"/>
-      <c r="D3" s="57"/>
-      <c r="E3" s="57"/>
-      <c r="F3" s="57"/>
-      <c r="G3" s="57" t="s">
+      <c r="B3" s="92" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="92"/>
+      <c r="D3" s="92"/>
+      <c r="E3" s="92"/>
+      <c r="F3" s="92"/>
+      <c r="G3" s="92" t="s">
         <v>1</v>
       </c>
-      <c r="H3" s="57"/>
-      <c r="I3" s="57"/>
-      <c r="J3" s="57"/>
-      <c r="K3" s="57"/>
-      <c r="L3" s="57" t="s">
+      <c r="H3" s="92"/>
+      <c r="I3" s="92"/>
+      <c r="J3" s="92"/>
+      <c r="K3" s="92"/>
+      <c r="L3" s="92" t="s">
         <v>2</v>
       </c>
-      <c r="M3" s="57"/>
-      <c r="N3" s="57"/>
-      <c r="O3" s="57"/>
-      <c r="P3" s="57"/>
-      <c r="Q3" s="57"/>
-      <c r="R3" s="58" t="s">
+      <c r="M3" s="92"/>
+      <c r="N3" s="92"/>
+      <c r="O3" s="92"/>
+      <c r="P3" s="92"/>
+      <c r="Q3" s="92"/>
+      <c r="R3" s="93" t="s">
         <v>3</v>
       </c>
-      <c r="S3" s="58"/>
-      <c r="T3" s="58"/>
-      <c r="U3" s="59" t="s">
+      <c r="S3" s="93"/>
+      <c r="T3" s="93"/>
+      <c r="U3" s="94" t="s">
         <v>4</v>
       </c>
-      <c r="V3" s="59"/>
-      <c r="W3" s="59"/>
-      <c r="X3" s="58" t="s">
+      <c r="V3" s="94"/>
+      <c r="W3" s="94"/>
+      <c r="X3" s="93" t="s">
         <v>5</v>
       </c>
-      <c r="Y3" s="58"/>
-      <c r="Z3" s="60">
+      <c r="Y3" s="93"/>
+      <c r="Z3" s="95">
         <f>Cadastro!G2</f>
         <v>2026</v>
       </c>
-      <c r="AA3" s="60"/>
+      <c r="AA3" s="95"/>
       <c r="AB3" s="4"/>
       <c r="AD3" s="1">
         <f>IF($U$3="Ano",12,AD1)</f>
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:60" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:60" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2"/>
-      <c r="B4" s="61">
+      <c r="B4" s="96">
         <f>BC18</f>
         <v>0</v>
       </c>
-      <c r="C4" s="61"/>
-      <c r="D4" s="61"/>
-      <c r="E4" s="61"/>
-      <c r="F4" s="61"/>
-      <c r="G4" s="61">
+      <c r="C4" s="96"/>
+      <c r="D4" s="96"/>
+      <c r="E4" s="96"/>
+      <c r="F4" s="96"/>
+      <c r="G4" s="96">
         <f>BC20</f>
-        <v>316349.37333333329</v>
-      </c>
-      <c r="H4" s="61"/>
-      <c r="I4" s="61"/>
-      <c r="J4" s="61"/>
-      <c r="K4" s="61"/>
-      <c r="L4" s="62">
+        <v>319728.86333333328</v>
+      </c>
+      <c r="H4" s="96"/>
+      <c r="I4" s="96"/>
+      <c r="J4" s="96"/>
+      <c r="K4" s="96"/>
+      <c r="L4" s="97">
         <f>BC18-BC20</f>
-        <v>-316349.37333333329</v>
-      </c>
-      <c r="M4" s="62"/>
-      <c r="N4" s="62"/>
-      <c r="O4" s="62"/>
-      <c r="P4" s="62"/>
-      <c r="Q4" s="62"/>
-      <c r="R4" s="58"/>
-      <c r="S4" s="58"/>
-      <c r="T4" s="58"/>
-      <c r="U4" s="59"/>
-      <c r="V4" s="59"/>
-      <c r="W4" s="59"/>
-      <c r="X4" s="58"/>
-      <c r="Y4" s="58"/>
-      <c r="Z4" s="60"/>
-      <c r="AA4" s="60"/>
+        <v>-319728.86333333328</v>
+      </c>
+      <c r="M4" s="97"/>
+      <c r="N4" s="97"/>
+      <c r="O4" s="97"/>
+      <c r="P4" s="97"/>
+      <c r="Q4" s="97"/>
+      <c r="R4" s="93"/>
+      <c r="S4" s="93"/>
+      <c r="T4" s="93"/>
+      <c r="U4" s="94"/>
+      <c r="V4" s="94"/>
+      <c r="W4" s="94"/>
+      <c r="X4" s="93"/>
+      <c r="Y4" s="93"/>
+      <c r="Z4" s="95"/>
+      <c r="AA4" s="95"/>
       <c r="AB4" s="4"/>
     </row>
-    <row r="5" spans="1:60" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:60" ht="6.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4"/>
       <c r="B5" s="4"/>
       <c r="C5" s="4"/>
@@ -4320,60 +4304,60 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:60" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:60" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4"/>
-      <c r="B6" s="67" t="s">
+      <c r="B6" s="90" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="67"/>
-      <c r="D6" s="63" t="s">
+      <c r="C6" s="90"/>
+      <c r="D6" s="86" t="s">
         <v>14</v>
       </c>
-      <c r="E6" s="63"/>
-      <c r="F6" s="63" t="s">
+      <c r="E6" s="86"/>
+      <c r="F6" s="86" t="s">
         <v>15</v>
       </c>
-      <c r="G6" s="63"/>
-      <c r="H6" s="63" t="s">
+      <c r="G6" s="86"/>
+      <c r="H6" s="86" t="s">
         <v>16</v>
       </c>
-      <c r="I6" s="63"/>
-      <c r="J6" s="63" t="s">
+      <c r="I6" s="86"/>
+      <c r="J6" s="86" t="s">
         <v>17</v>
       </c>
-      <c r="K6" s="63"/>
-      <c r="L6" s="63" t="s">
+      <c r="K6" s="86"/>
+      <c r="L6" s="86" t="s">
         <v>18</v>
       </c>
-      <c r="M6" s="63"/>
-      <c r="N6" s="63" t="s">
+      <c r="M6" s="86"/>
+      <c r="N6" s="86" t="s">
         <v>19</v>
       </c>
-      <c r="O6" s="63"/>
-      <c r="P6" s="63" t="s">
+      <c r="O6" s="86"/>
+      <c r="P6" s="86" t="s">
         <v>20</v>
       </c>
-      <c r="Q6" s="63"/>
-      <c r="R6" s="63" t="s">
+      <c r="Q6" s="86"/>
+      <c r="R6" s="86" t="s">
         <v>21</v>
       </c>
-      <c r="S6" s="63"/>
-      <c r="T6" s="63" t="s">
+      <c r="S6" s="86"/>
+      <c r="T6" s="86" t="s">
         <v>22</v>
       </c>
-      <c r="U6" s="63"/>
-      <c r="V6" s="63" t="s">
+      <c r="U6" s="86"/>
+      <c r="V6" s="86" t="s">
         <v>23</v>
       </c>
-      <c r="W6" s="63"/>
-      <c r="X6" s="63" t="s">
+      <c r="W6" s="86"/>
+      <c r="X6" s="86" t="s">
         <v>24</v>
       </c>
-      <c r="Y6" s="63"/>
-      <c r="Z6" s="63" t="s">
+      <c r="Y6" s="86"/>
+      <c r="Z6" s="86" t="s">
         <v>25</v>
       </c>
-      <c r="AA6" s="63"/>
+      <c r="AA6" s="86"/>
       <c r="AB6" s="4"/>
       <c r="AE6" s="1" t="s">
         <v>14</v>
@@ -4452,7 +4436,7 @@
       </c>
       <c r="BC6" s="1">
         <f>SUMPRODUCT((Lançamentos!$C$3:$N$3&gt;=$AD$1)*(Lançamentos!$C$3:$N$3&lt;=$AD$3)*Lançamentos!$C$23:$N$23)</f>
-        <v>316349.37333333329</v>
+        <v>319728.86333333328</v>
       </c>
       <c r="BE6" s="1" t="str">
         <f t="shared" ref="BE6:BE17" si="7">AE6</f>
@@ -4471,7 +4455,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" spans="1:60" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:60" ht="6.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4"/>
       <c r="B7" s="4"/>
       <c r="C7" s="4"/>
@@ -4596,47 +4580,47 @@
         <v/>
       </c>
     </row>
-    <row r="8" spans="1:60" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:60" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4"/>
-      <c r="B8" s="64" t="str">
+      <c r="B8" s="87" t="str">
         <f>"Realizado · "&amp;$BC$14</f>
         <v>Realizado · Ano 2026</v>
       </c>
-      <c r="C8" s="64"/>
-      <c r="D8" s="64"/>
-      <c r="E8" s="64"/>
-      <c r="F8" s="64" t="s">
+      <c r="C8" s="87"/>
+      <c r="D8" s="87"/>
+      <c r="E8" s="87"/>
+      <c r="F8" s="87" t="s">
         <v>26</v>
       </c>
-      <c r="G8" s="64"/>
-      <c r="H8" s="64"/>
-      <c r="I8" s="64"/>
-      <c r="J8" s="65" t="s">
+      <c r="G8" s="87"/>
+      <c r="H8" s="87"/>
+      <c r="I8" s="87"/>
+      <c r="J8" s="88" t="s">
         <v>27</v>
       </c>
-      <c r="K8" s="65"/>
-      <c r="L8" s="65"/>
-      <c r="M8" s="65"/>
-      <c r="N8" s="65" t="s">
+      <c r="K8" s="88"/>
+      <c r="L8" s="88"/>
+      <c r="M8" s="88"/>
+      <c r="N8" s="88" t="s">
         <v>28</v>
       </c>
-      <c r="O8" s="65"/>
-      <c r="P8" s="65"/>
-      <c r="Q8" s="65"/>
-      <c r="R8" s="66" t="s">
+      <c r="O8" s="88"/>
+      <c r="P8" s="88"/>
+      <c r="Q8" s="88"/>
+      <c r="R8" s="89" t="s">
         <v>29</v>
       </c>
-      <c r="S8" s="66"/>
-      <c r="T8" s="66"/>
-      <c r="U8" s="66"/>
-      <c r="V8" s="66"/>
-      <c r="W8" s="66" t="s">
+      <c r="S8" s="89"/>
+      <c r="T8" s="89"/>
+      <c r="U8" s="89"/>
+      <c r="V8" s="89"/>
+      <c r="W8" s="89" t="s">
         <v>30</v>
       </c>
-      <c r="X8" s="66"/>
-      <c r="Y8" s="66"/>
-      <c r="Z8" s="66"/>
-      <c r="AA8" s="66"/>
+      <c r="X8" s="89"/>
+      <c r="Y8" s="89"/>
+      <c r="Z8" s="89"/>
+      <c r="AA8" s="89"/>
       <c r="AB8" s="4"/>
       <c r="AE8" s="1" t="s">
         <v>16</v>
@@ -4734,52 +4718,52 @@
         <v/>
       </c>
     </row>
-    <row r="9" spans="1:60" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:60" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4"/>
-      <c r="B9" s="68">
+      <c r="B9" s="74">
         <f>BC6</f>
-        <v>316349.37333333329</v>
-      </c>
-      <c r="C9" s="68"/>
-      <c r="D9" s="68"/>
-      <c r="E9" s="68"/>
-      <c r="F9" s="69">
+        <v>319728.86333333328</v>
+      </c>
+      <c r="C9" s="74"/>
+      <c r="D9" s="74"/>
+      <c r="E9" s="74"/>
+      <c r="F9" s="75">
         <f>IF(BC15=0,0,BC6/BC15-1)</f>
-        <v>3.4574705534529127E-3</v>
-      </c>
-      <c r="G9" s="69"/>
-      <c r="H9" s="69"/>
-      <c r="I9" s="69"/>
-      <c r="J9" s="70">
+        <v>1.4177183544910044E-2</v>
+      </c>
+      <c r="G9" s="75"/>
+      <c r="H9" s="75"/>
+      <c r="I9" s="75"/>
+      <c r="J9" s="76">
         <f>IF(BC10=0,0,BC9/BC10)</f>
         <v>0</v>
       </c>
-      <c r="K9" s="70"/>
-      <c r="L9" s="70"/>
-      <c r="M9" s="70"/>
-      <c r="N9" s="71">
+      <c r="K9" s="76"/>
+      <c r="L9" s="76"/>
+      <c r="M9" s="76"/>
+      <c r="N9" s="77">
         <f>IF(BC11=0,0,BC9/BC11)</f>
-        <v>39543.671666666662</v>
-      </c>
-      <c r="O9" s="71"/>
-      <c r="P9" s="71"/>
-      <c r="Q9" s="71"/>
-      <c r="R9" s="72">
+        <v>35525.429259259254</v>
+      </c>
+      <c r="O9" s="77"/>
+      <c r="P9" s="77"/>
+      <c r="Q9" s="77"/>
+      <c r="R9" s="78">
         <f>IF(BC6&gt;0,BC12/BC6,IF(BC7=0,0,BC13/BC7))</f>
-        <v>0.36394723588936673</v>
-      </c>
-      <c r="S9" s="72"/>
-      <c r="T9" s="72"/>
-      <c r="U9" s="72"/>
-      <c r="V9" s="72"/>
-      <c r="W9" s="73" t="str">
+        <v>0.36010036378844706</v>
+      </c>
+      <c r="S9" s="78"/>
+      <c r="T9" s="78"/>
+      <c r="U9" s="78"/>
+      <c r="V9" s="78"/>
+      <c r="W9" s="79" t="str">
         <f>IF($U$3="Ano",COUNTIF(Lançamentos!$C$25:$N$25,"Completo")&amp;" de 12 meses",INDEX(Lançamentos!$C$25:$N$25,$AD$1))</f>
         <v>0 de 12 meses</v>
       </c>
-      <c r="X9" s="73"/>
-      <c r="Y9" s="73"/>
-      <c r="Z9" s="73"/>
-      <c r="AA9" s="73"/>
+      <c r="X9" s="79"/>
+      <c r="Y9" s="79"/>
+      <c r="Z9" s="79"/>
+      <c r="AA9" s="79"/>
       <c r="AB9" s="4"/>
       <c r="AE9" s="1" t="s">
         <v>17</v>
@@ -4834,7 +4818,7 @@
       </c>
       <c r="AU9" s="1">
         <f t="shared" si="2"/>
-        <v>27035.919999999991</v>
+        <v>30415.409999999989</v>
       </c>
       <c r="AV9" s="1">
         <f t="shared" si="3"/>
@@ -4858,7 +4842,7 @@
       </c>
       <c r="BC9" s="1">
         <f>SUMPRODUCT((Lançamentos!$C$3:$N$3&lt;=$AD$3)*Lançamentos!$C$23:$N$23)</f>
-        <v>316349.37333333329</v>
+        <v>319728.86333333328</v>
       </c>
       <c r="BE9" s="1" t="str">
         <f t="shared" si="7"/>
@@ -4877,34 +4861,34 @@
         <v/>
       </c>
     </row>
-    <row r="10" spans="1:60" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:60" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4"/>
-      <c r="B10" s="68"/>
-      <c r="C10" s="68"/>
-      <c r="D10" s="68"/>
-      <c r="E10" s="68"/>
-      <c r="F10" s="69"/>
-      <c r="G10" s="69"/>
-      <c r="H10" s="69"/>
-      <c r="I10" s="69"/>
-      <c r="J10" s="70"/>
-      <c r="K10" s="70"/>
-      <c r="L10" s="70"/>
-      <c r="M10" s="70"/>
-      <c r="N10" s="71"/>
-      <c r="O10" s="71"/>
-      <c r="P10" s="71"/>
-      <c r="Q10" s="71"/>
-      <c r="R10" s="72"/>
-      <c r="S10" s="72"/>
-      <c r="T10" s="72"/>
-      <c r="U10" s="72"/>
-      <c r="V10" s="72"/>
-      <c r="W10" s="73"/>
-      <c r="X10" s="73"/>
-      <c r="Y10" s="73"/>
-      <c r="Z10" s="73"/>
-      <c r="AA10" s="73"/>
+      <c r="B10" s="74"/>
+      <c r="C10" s="74"/>
+      <c r="D10" s="74"/>
+      <c r="E10" s="74"/>
+      <c r="F10" s="75"/>
+      <c r="G10" s="75"/>
+      <c r="H10" s="75"/>
+      <c r="I10" s="75"/>
+      <c r="J10" s="76"/>
+      <c r="K10" s="76"/>
+      <c r="L10" s="76"/>
+      <c r="M10" s="76"/>
+      <c r="N10" s="77"/>
+      <c r="O10" s="77"/>
+      <c r="P10" s="77"/>
+      <c r="Q10" s="77"/>
+      <c r="R10" s="78"/>
+      <c r="S10" s="78"/>
+      <c r="T10" s="78"/>
+      <c r="U10" s="78"/>
+      <c r="V10" s="78"/>
+      <c r="W10" s="79"/>
+      <c r="X10" s="79"/>
+      <c r="Y10" s="79"/>
+      <c r="Z10" s="79"/>
+      <c r="AA10" s="79"/>
       <c r="AB10" s="4"/>
       <c r="AE10" s="1" t="s">
         <v>18</v>
@@ -5002,64 +4986,64 @@
         <v/>
       </c>
     </row>
-    <row r="11" spans="1:60" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:60" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4"/>
-      <c r="B11" s="74" t="s">
+      <c r="B11" s="80" t="s">
         <v>7</v>
       </c>
-      <c r="C11" s="74"/>
-      <c r="D11" s="75">
+      <c r="C11" s="80"/>
+      <c r="D11" s="81">
         <f>BC7</f>
         <v>315259.37333333329</v>
       </c>
-      <c r="E11" s="75"/>
-      <c r="F11" s="74" t="s">
+      <c r="E11" s="81"/>
+      <c r="F11" s="80" t="s">
         <v>31</v>
       </c>
-      <c r="G11" s="74"/>
-      <c r="H11" s="76">
+      <c r="G11" s="80"/>
+      <c r="H11" s="82">
         <f>BC6-BC15</f>
-        <v>1090</v>
-      </c>
-      <c r="I11" s="76"/>
-      <c r="J11" s="77" t="s">
+        <v>4469.4899999999907</v>
+      </c>
+      <c r="I11" s="82"/>
+      <c r="J11" s="83" t="s">
         <v>32</v>
       </c>
-      <c r="K11" s="77"/>
-      <c r="L11" s="75">
+      <c r="K11" s="83"/>
+      <c r="L11" s="81">
         <f>BC10-BC9</f>
-        <v>-316349.37333333329</v>
-      </c>
-      <c r="M11" s="75"/>
-      <c r="N11" s="77" t="s">
+        <v>-319728.86333333328</v>
+      </c>
+      <c r="M11" s="81"/>
+      <c r="N11" s="83" t="s">
         <v>33</v>
       </c>
-      <c r="O11" s="77"/>
-      <c r="P11" s="75">
+      <c r="O11" s="83"/>
+      <c r="P11" s="81">
         <f>Cadastro!H23</f>
         <v>15577.880833333333</v>
       </c>
-      <c r="Q11" s="75"/>
-      <c r="R11" s="78" t="s">
+      <c r="Q11" s="81"/>
+      <c r="R11" s="84" t="s">
         <v>34</v>
       </c>
-      <c r="S11" s="78"/>
-      <c r="T11" s="75">
+      <c r="S11" s="84"/>
+      <c r="T11" s="81">
         <f>IF(BC6&gt;0,BC12,BC13)</f>
         <v>115134.48</v>
       </c>
-      <c r="U11" s="75"/>
-      <c r="V11" s="75"/>
-      <c r="W11" s="78" t="s">
+      <c r="U11" s="81"/>
+      <c r="V11" s="81"/>
+      <c r="W11" s="84" t="s">
         <v>35</v>
       </c>
-      <c r="X11" s="78"/>
-      <c r="Y11" s="79" t="str">
+      <c r="X11" s="84"/>
+      <c r="Y11" s="85" t="str">
         <f>IF($U$3="Ano",BC11&amp;" c/ dados",INDEX(Lançamentos!$C$24:$N$24,$AD$1)&amp;"/"&amp;COUNTA(Cadastro!$B$5:$B$22))</f>
-        <v>8 c/ dados</v>
-      </c>
-      <c r="Z11" s="79"/>
-      <c r="AA11" s="79"/>
+        <v>9 c/ dados</v>
+      </c>
+      <c r="Z11" s="85"/>
+      <c r="AA11" s="85"/>
       <c r="AB11" s="4"/>
       <c r="AE11" s="1" t="s">
         <v>19</v>
@@ -5138,7 +5122,7 @@
       </c>
       <c r="BC11" s="1">
         <f>SUMPRODUCT((Lançamentos!$C$3:$N$3&lt;=$AD$3)*(Lançamentos!$C$24:$N$24&gt;0))</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="BE11" s="1" t="str">
         <f t="shared" si="7"/>
@@ -5157,7 +5141,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" spans="1:60" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:60" ht="6.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4"/>
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
@@ -5266,39 +5250,39 @@
         <v/>
       </c>
     </row>
-    <row r="13" spans="1:60" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:60" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="4"/>
-      <c r="B13" s="80" t="s">
+      <c r="B13" s="71" t="s">
         <v>36</v>
       </c>
-      <c r="C13" s="80"/>
-      <c r="D13" s="80"/>
-      <c r="E13" s="80"/>
-      <c r="F13" s="80"/>
-      <c r="G13" s="80"/>
-      <c r="H13" s="80"/>
-      <c r="I13" s="80"/>
-      <c r="J13" s="80"/>
-      <c r="K13" s="80"/>
-      <c r="L13" s="80"/>
-      <c r="M13" s="80"/>
-      <c r="N13" s="80"/>
-      <c r="O13" s="80"/>
-      <c r="P13" s="80"/>
-      <c r="Q13" s="80"/>
-      <c r="R13" s="80" t="str">
+      <c r="C13" s="71"/>
+      <c r="D13" s="71"/>
+      <c r="E13" s="71"/>
+      <c r="F13" s="71"/>
+      <c r="G13" s="71"/>
+      <c r="H13" s="71"/>
+      <c r="I13" s="71"/>
+      <c r="J13" s="71"/>
+      <c r="K13" s="71"/>
+      <c r="L13" s="71"/>
+      <c r="M13" s="71"/>
+      <c r="N13" s="71"/>
+      <c r="O13" s="71"/>
+      <c r="P13" s="71"/>
+      <c r="Q13" s="71"/>
+      <c r="R13" s="71" t="str">
         <f>"Por categoria · "&amp;$BC$14</f>
         <v>Por categoria · Ano 2026</v>
       </c>
-      <c r="S13" s="80"/>
-      <c r="T13" s="80"/>
-      <c r="U13" s="80"/>
-      <c r="V13" s="80"/>
-      <c r="W13" s="80"/>
-      <c r="X13" s="80"/>
-      <c r="Y13" s="80"/>
-      <c r="Z13" s="80"/>
-      <c r="AA13" s="80"/>
+      <c r="S13" s="71"/>
+      <c r="T13" s="71"/>
+      <c r="U13" s="71"/>
+      <c r="V13" s="71"/>
+      <c r="W13" s="71"/>
+      <c r="X13" s="71"/>
+      <c r="Y13" s="71"/>
+      <c r="Z13" s="71"/>
+      <c r="AA13" s="71"/>
       <c r="AB13" s="4"/>
       <c r="AE13" s="1" t="s">
         <v>21</v>
@@ -5380,7 +5364,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" spans="1:60" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:60" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="4"/>
       <c r="B14" s="7"/>
       <c r="C14" s="8"/>
@@ -5416,9 +5400,9 @@
         <f>Orçado!K23</f>
         <v>0</v>
       </c>
-      <c r="AG14" s="5" t="str">
+      <c r="AG14" s="5">
         <f>IF(AI14=0,"",IF(AND($U$3&lt;&gt;"Ano",9=$AD$1),"",Lançamentos!K23))</f>
-        <v/>
+        <v>3379.49</v>
       </c>
       <c r="AH14" s="1" t="str">
         <f>IF(AND($U$3&lt;&gt;"Ano",9=$AD$1,AI14=1),Lançamentos!K23,"")</f>
@@ -5426,7 +5410,7 @@
       </c>
       <c r="AI14" s="1">
         <f>IF(Lançamentos!K24&gt;0,1,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AL14" s="1" t="str">
         <f>Lançamentos!A13</f>
@@ -5480,16 +5464,16 @@
         <f>IF(Faturamento!K17=0,"",Faturamento!K16)</f>
         <v/>
       </c>
-      <c r="BG14" s="5" t="str">
+      <c r="BG14" s="5">
         <f>IF(Lançamentos!K24=0,"",Lançamentos!K23)</f>
-        <v/>
+        <v>3379.49</v>
       </c>
       <c r="BH14" s="1" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
-    <row r="15" spans="1:60" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:60" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="4"/>
       <c r="B15" s="7"/>
       <c r="C15" s="8"/>
@@ -5598,7 +5582,7 @@
         <v/>
       </c>
     </row>
-    <row r="16" spans="1:60" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:60" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="4"/>
       <c r="B16" s="7"/>
       <c r="C16" s="8"/>
@@ -5687,7 +5671,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" spans="1:60" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:60" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="4"/>
       <c r="B17" s="7"/>
       <c r="C17" s="8"/>
@@ -5780,7 +5764,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" spans="1:60" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:60" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="4"/>
       <c r="B18" s="7"/>
       <c r="C18" s="8"/>
@@ -5838,7 +5822,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:60" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:60" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="4"/>
       <c r="B19" s="7"/>
       <c r="C19" s="8"/>
@@ -5896,7 +5880,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:60" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:60" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="4"/>
       <c r="B20" s="7"/>
       <c r="C20" s="8"/>
@@ -5951,10 +5935,10 @@
       </c>
       <c r="BC20" s="1">
         <f>SUM(Lançamentos!$C$23:$N$23)</f>
-        <v>316349.37333333329</v>
-      </c>
-    </row>
-    <row r="21" spans="1:60" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+        <v>319728.86333333328</v>
+      </c>
+    </row>
+    <row r="21" spans="1:60" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="4"/>
       <c r="B21" s="7"/>
       <c r="C21" s="8"/>
@@ -6008,7 +5992,7 @@
         <v>112281.31228122099</v>
       </c>
     </row>
-    <row r="22" spans="1:60" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:60" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="4"/>
       <c r="B22" s="7"/>
       <c r="C22" s="8"/>
@@ -6062,7 +6046,7 @@
         <v>4198.0041980219994</v>
       </c>
     </row>
-    <row r="23" spans="1:60" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:60" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="4"/>
       <c r="B23" s="7"/>
       <c r="C23" s="8"/>
@@ -6116,7 +6100,7 @@
         <v>3714.4970478496616</v>
       </c>
     </row>
-    <row r="24" spans="1:60" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:60" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="4"/>
       <c r="B24" s="7"/>
       <c r="C24" s="8"/>
@@ -6159,7 +6143,7 @@
       </c>
       <c r="AO24" s="1">
         <f>IF(AL24="","",SUMPRODUCT((Lançamentos!$C$3:$N$3&gt;=$AD$1)*(Lançamentos!$C$3:$N$3&lt;=$AD$3)*Lançamentos!$C20:$N20))</f>
-        <v>27035.919999999991</v>
+        <v>30415.409999999989</v>
       </c>
       <c r="AP24" s="1">
         <f>IF(AL24="","",IF($BC$8&gt;0,SUMPRODUCT((Lançamentos!$C$3:$N$3&gt;=$AD$1)*(Lançamentos!$C$3:$N$3&lt;=$AD$3)*(Lançamentos!$C$24:$N$24&gt;0)*Orçado!$C20:$N20),AN24))</f>
@@ -6167,10 +6151,10 @@
       </c>
       <c r="AQ24" s="1">
         <f t="shared" si="0"/>
-        <v>27035.947035943991</v>
-      </c>
-    </row>
-    <row r="25" spans="1:60" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+        <v>30415.437035943989</v>
+      </c>
+    </row>
+    <row r="25" spans="1:60" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="4"/>
       <c r="B25" s="7"/>
       <c r="C25" s="8"/>
@@ -6224,7 +6208,7 @@
         <v>488.00048802500004</v>
       </c>
     </row>
-    <row r="26" spans="1:60" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:60" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="4"/>
       <c r="B26" s="7"/>
       <c r="C26" s="8"/>
@@ -6254,7 +6238,7 @@
       <c r="AA26" s="9"/>
       <c r="AB26" s="4"/>
     </row>
-    <row r="27" spans="1:60" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:60" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="4"/>
       <c r="B27" s="7"/>
       <c r="C27" s="8"/>
@@ -6284,7 +6268,7 @@
       <c r="AA27" s="9"/>
       <c r="AB27" s="4"/>
     </row>
-    <row r="28" spans="1:60" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:60" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="4"/>
       <c r="B28" s="10"/>
       <c r="C28" s="11"/>
@@ -6314,7 +6298,7 @@
       <c r="AA28" s="12"/>
       <c r="AB28" s="4"/>
     </row>
-    <row r="29" spans="1:60" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:60" ht="6.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="4"/>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -6344,43 +6328,43 @@
       <c r="AA29" s="4"/>
       <c r="AB29" s="4"/>
     </row>
-    <row r="30" spans="1:60" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:60" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="4"/>
-      <c r="B30" s="80" t="str">
+      <c r="B30" s="71" t="str">
         <f>"Por despesa · "&amp;$BC$14</f>
         <v>Por despesa · Ano 2026</v>
       </c>
-      <c r="C30" s="80"/>
-      <c r="D30" s="80"/>
-      <c r="E30" s="80"/>
-      <c r="F30" s="80"/>
-      <c r="G30" s="80"/>
-      <c r="H30" s="80"/>
-      <c r="I30" s="80"/>
-      <c r="J30" s="80"/>
-      <c r="K30" s="80"/>
-      <c r="L30" s="80"/>
-      <c r="M30" s="80"/>
-      <c r="N30" s="80"/>
-      <c r="O30" s="80" t="str">
+      <c r="C30" s="71"/>
+      <c r="D30" s="71"/>
+      <c r="E30" s="71"/>
+      <c r="F30" s="71"/>
+      <c r="G30" s="71"/>
+      <c r="H30" s="71"/>
+      <c r="I30" s="71"/>
+      <c r="J30" s="71"/>
+      <c r="K30" s="71"/>
+      <c r="L30" s="71"/>
+      <c r="M30" s="71"/>
+      <c r="N30" s="71"/>
+      <c r="O30" s="71" t="str">
         <f>"Detalhe · "&amp;$BC$14</f>
         <v>Detalhe · Ano 2026</v>
       </c>
-      <c r="P30" s="80"/>
-      <c r="Q30" s="80"/>
-      <c r="R30" s="80"/>
-      <c r="S30" s="80"/>
-      <c r="T30" s="80"/>
-      <c r="U30" s="80"/>
-      <c r="V30" s="80"/>
-      <c r="W30" s="80"/>
-      <c r="X30" s="80"/>
-      <c r="Y30" s="80"/>
-      <c r="Z30" s="80"/>
-      <c r="AA30" s="80"/>
+      <c r="P30" s="71"/>
+      <c r="Q30" s="71"/>
+      <c r="R30" s="71"/>
+      <c r="S30" s="71"/>
+      <c r="T30" s="71"/>
+      <c r="U30" s="71"/>
+      <c r="V30" s="71"/>
+      <c r="W30" s="71"/>
+      <c r="X30" s="71"/>
+      <c r="Y30" s="71"/>
+      <c r="Z30" s="71"/>
+      <c r="AA30" s="71"/>
       <c r="AB30" s="4"/>
     </row>
-    <row r="31" spans="1:60" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:60" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="4"/>
       <c r="B31" s="7"/>
       <c r="C31" s="8"/>
@@ -6410,7 +6394,7 @@
       <c r="AA31" s="9"/>
       <c r="AB31" s="4"/>
     </row>
-    <row r="32" spans="1:60" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:60" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="4"/>
       <c r="B32" s="7"/>
       <c r="C32" s="8"/>
@@ -6425,30 +6409,30 @@
       <c r="L32" s="8"/>
       <c r="M32" s="8"/>
       <c r="N32" s="9"/>
-      <c r="O32" s="81" t="s">
+      <c r="O32" s="72" t="s">
         <v>12</v>
       </c>
-      <c r="P32" s="81"/>
-      <c r="Q32" s="81"/>
-      <c r="R32" s="81"/>
-      <c r="S32" s="81"/>
-      <c r="T32" s="82" t="s">
+      <c r="P32" s="72"/>
+      <c r="Q32" s="72"/>
+      <c r="R32" s="72"/>
+      <c r="S32" s="72"/>
+      <c r="T32" s="73" t="s">
         <v>7</v>
       </c>
-      <c r="U32" s="82"/>
-      <c r="V32" s="82"/>
-      <c r="W32" s="82" t="s">
+      <c r="U32" s="73"/>
+      <c r="V32" s="73"/>
+      <c r="W32" s="73" t="s">
         <v>8</v>
       </c>
-      <c r="X32" s="82"/>
-      <c r="Y32" s="82"/>
-      <c r="Z32" s="82" t="s">
+      <c r="X32" s="73"/>
+      <c r="Y32" s="73"/>
+      <c r="Z32" s="73" t="s">
         <v>37</v>
       </c>
-      <c r="AA32" s="82"/>
+      <c r="AA32" s="73"/>
       <c r="AB32" s="4"/>
     </row>
-    <row r="33" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="4"/>
       <c r="B33" s="7"/>
       <c r="C33" s="8"/>
@@ -6463,34 +6447,34 @@
       <c r="L33" s="8"/>
       <c r="M33" s="8"/>
       <c r="N33" s="9"/>
-      <c r="O33" s="83" t="str">
+      <c r="O33" s="67" t="str">
         <f t="shared" ref="O33:O42" si="9">AT6</f>
         <v>Funcionários</v>
       </c>
-      <c r="P33" s="83"/>
-      <c r="Q33" s="83"/>
-      <c r="R33" s="83"/>
-      <c r="S33" s="83"/>
-      <c r="T33" s="84">
+      <c r="P33" s="67"/>
+      <c r="Q33" s="67"/>
+      <c r="R33" s="67"/>
+      <c r="S33" s="67"/>
+      <c r="T33" s="68">
         <f t="shared" ref="T33:T41" si="10">IF(AT6="","",AV6)</f>
         <v>113702.48</v>
       </c>
-      <c r="U33" s="84"/>
-      <c r="V33" s="84"/>
-      <c r="W33" s="85">
+      <c r="U33" s="68"/>
+      <c r="V33" s="68"/>
+      <c r="W33" s="69">
         <f t="shared" ref="W33:W42" si="11">IF(AT6="","",AU6)</f>
         <v>113702.48</v>
       </c>
-      <c r="X33" s="85"/>
-      <c r="Y33" s="85"/>
-      <c r="Z33" s="86">
+      <c r="X33" s="69"/>
+      <c r="Y33" s="69"/>
+      <c r="Z33" s="70">
         <f t="shared" ref="Z33:Z42" si="12">IF(OR(AT6="",N(AU6)=0,N(AV6)=0),"",AU6/AV6-1)</f>
         <v>0</v>
       </c>
-      <c r="AA33" s="86"/>
+      <c r="AA33" s="70"/>
       <c r="AB33" s="4"/>
     </row>
-    <row r="34" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="4"/>
       <c r="B34" s="7"/>
       <c r="C34" s="8"/>
@@ -6505,34 +6489,34 @@
       <c r="L34" s="8"/>
       <c r="M34" s="8"/>
       <c r="N34" s="9"/>
-      <c r="O34" s="83" t="str">
+      <c r="O34" s="67" t="str">
         <f t="shared" si="9"/>
         <v>Tubete</v>
       </c>
-      <c r="P34" s="83"/>
-      <c r="Q34" s="83"/>
-      <c r="R34" s="83"/>
-      <c r="S34" s="83"/>
-      <c r="T34" s="84">
+      <c r="P34" s="67"/>
+      <c r="Q34" s="67"/>
+      <c r="R34" s="67"/>
+      <c r="S34" s="67"/>
+      <c r="T34" s="68">
         <f t="shared" si="10"/>
         <v>112281.2</v>
       </c>
-      <c r="U34" s="84"/>
-      <c r="V34" s="84"/>
-      <c r="W34" s="85">
+      <c r="U34" s="68"/>
+      <c r="V34" s="68"/>
+      <c r="W34" s="69">
         <f t="shared" si="11"/>
         <v>112281.2</v>
       </c>
-      <c r="X34" s="85"/>
-      <c r="Y34" s="85"/>
-      <c r="Z34" s="86">
+      <c r="X34" s="69"/>
+      <c r="Y34" s="69"/>
+      <c r="Z34" s="70">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="AA34" s="86"/>
+      <c r="AA34" s="70"/>
       <c r="AB34" s="4"/>
     </row>
-    <row r="35" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="4"/>
       <c r="B35" s="7"/>
       <c r="C35" s="8"/>
@@ -6547,34 +6531,34 @@
       <c r="L35" s="8"/>
       <c r="M35" s="8"/>
       <c r="N35" s="9"/>
-      <c r="O35" s="83" t="str">
+      <c r="O35" s="67" t="str">
         <f t="shared" si="9"/>
         <v>Combustivel</v>
       </c>
-      <c r="P35" s="83"/>
-      <c r="Q35" s="83"/>
-      <c r="R35" s="83"/>
-      <c r="S35" s="83"/>
-      <c r="T35" s="84">
+      <c r="P35" s="67"/>
+      <c r="Q35" s="67"/>
+      <c r="R35" s="67"/>
+      <c r="S35" s="67"/>
+      <c r="T35" s="68">
         <f t="shared" si="10"/>
         <v>30733.02</v>
       </c>
-      <c r="U35" s="84"/>
-      <c r="V35" s="84"/>
-      <c r="W35" s="85">
+      <c r="U35" s="68"/>
+      <c r="V35" s="68"/>
+      <c r="W35" s="69">
         <f t="shared" si="11"/>
         <v>30733.02</v>
       </c>
-      <c r="X35" s="85"/>
-      <c r="Y35" s="85"/>
-      <c r="Z35" s="86">
+      <c r="X35" s="69"/>
+      <c r="Y35" s="69"/>
+      <c r="Z35" s="70">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="AA35" s="86"/>
+      <c r="AA35" s="70"/>
       <c r="AB35" s="4"/>
     </row>
-    <row r="36" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="4"/>
       <c r="B36" s="7"/>
       <c r="C36" s="8"/>
@@ -6589,34 +6573,34 @@
       <c r="L36" s="8"/>
       <c r="M36" s="8"/>
       <c r="N36" s="9"/>
-      <c r="O36" s="83" t="str">
+      <c r="O36" s="67" t="str">
         <f t="shared" si="9"/>
         <v>Parcela Caminhão</v>
       </c>
-      <c r="P36" s="83"/>
-      <c r="Q36" s="83"/>
-      <c r="R36" s="83"/>
-      <c r="S36" s="83"/>
-      <c r="T36" s="84">
+      <c r="P36" s="67"/>
+      <c r="Q36" s="67"/>
+      <c r="R36" s="67"/>
+      <c r="S36" s="67"/>
+      <c r="T36" s="68">
         <f t="shared" si="10"/>
         <v>27035.919999999991</v>
       </c>
-      <c r="U36" s="84"/>
-      <c r="V36" s="84"/>
-      <c r="W36" s="85">
+      <c r="U36" s="68"/>
+      <c r="V36" s="68"/>
+      <c r="W36" s="69">
         <f t="shared" si="11"/>
-        <v>27035.919999999991</v>
-      </c>
-      <c r="X36" s="85"/>
-      <c r="Y36" s="85"/>
-      <c r="Z36" s="86">
+        <v>30415.409999999989</v>
+      </c>
+      <c r="X36" s="69"/>
+      <c r="Y36" s="69"/>
+      <c r="Z36" s="70">
         <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-      <c r="AA36" s="86"/>
+        <v>0.125</v>
+      </c>
+      <c r="AA36" s="70"/>
       <c r="AB36" s="4"/>
     </row>
-    <row r="37" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="4"/>
       <c r="B37" s="7"/>
       <c r="C37" s="8"/>
@@ -6631,34 +6615,34 @@
       <c r="L37" s="8"/>
       <c r="M37" s="8"/>
       <c r="N37" s="9"/>
-      <c r="O37" s="83" t="str">
+      <c r="O37" s="67" t="str">
         <f t="shared" si="9"/>
         <v>Manutenção Veicular (peças, servico, revisao, licenciamento)</v>
       </c>
-      <c r="P37" s="83"/>
-      <c r="Q37" s="83"/>
-      <c r="R37" s="83"/>
-      <c r="S37" s="83"/>
-      <c r="T37" s="84">
+      <c r="P37" s="67"/>
+      <c r="Q37" s="67"/>
+      <c r="R37" s="67"/>
+      <c r="S37" s="67"/>
+      <c r="T37" s="68">
         <f t="shared" si="10"/>
         <v>9533</v>
       </c>
-      <c r="U37" s="84"/>
-      <c r="V37" s="84"/>
-      <c r="W37" s="85">
+      <c r="U37" s="68"/>
+      <c r="V37" s="68"/>
+      <c r="W37" s="69">
         <f t="shared" si="11"/>
         <v>10623</v>
       </c>
-      <c r="X37" s="85"/>
-      <c r="Y37" s="85"/>
-      <c r="Z37" s="86">
+      <c r="X37" s="69"/>
+      <c r="Y37" s="69"/>
+      <c r="Z37" s="70">
         <f t="shared" si="12"/>
         <v>0.11433966222595204</v>
       </c>
-      <c r="AA37" s="86"/>
+      <c r="AA37" s="70"/>
       <c r="AB37" s="4"/>
     </row>
-    <row r="38" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="4"/>
       <c r="B38" s="7"/>
       <c r="C38" s="8"/>
@@ -6673,34 +6657,34 @@
       <c r="L38" s="8"/>
       <c r="M38" s="8"/>
       <c r="N38" s="9"/>
-      <c r="O38" s="83" t="str">
+      <c r="O38" s="67" t="str">
         <f t="shared" si="9"/>
         <v>Manutenção Predial</v>
       </c>
-      <c r="P38" s="83"/>
-      <c r="Q38" s="83"/>
-      <c r="R38" s="83"/>
-      <c r="S38" s="83"/>
-      <c r="T38" s="84">
+      <c r="P38" s="67"/>
+      <c r="Q38" s="67"/>
+      <c r="R38" s="67"/>
+      <c r="S38" s="67"/>
+      <c r="T38" s="68">
         <f t="shared" si="10"/>
         <v>4198</v>
       </c>
-      <c r="U38" s="84"/>
-      <c r="V38" s="84"/>
-      <c r="W38" s="85">
+      <c r="U38" s="68"/>
+      <c r="V38" s="68"/>
+      <c r="W38" s="69">
         <f t="shared" si="11"/>
         <v>4198</v>
       </c>
-      <c r="X38" s="85"/>
-      <c r="Y38" s="85"/>
-      <c r="Z38" s="86">
+      <c r="X38" s="69"/>
+      <c r="Y38" s="69"/>
+      <c r="Z38" s="70">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="AA38" s="86"/>
+      <c r="AA38" s="70"/>
       <c r="AB38" s="4"/>
     </row>
-    <row r="39" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="4"/>
       <c r="B39" s="7"/>
       <c r="C39" s="8"/>
@@ -6715,34 +6699,34 @@
       <c r="L39" s="8"/>
       <c r="M39" s="8"/>
       <c r="N39" s="9"/>
-      <c r="O39" s="83" t="str">
+      <c r="O39" s="67" t="str">
         <f t="shared" si="9"/>
         <v>Seguro do Caminhão</v>
       </c>
-      <c r="P39" s="83"/>
-      <c r="Q39" s="83"/>
-      <c r="R39" s="83"/>
-      <c r="S39" s="83"/>
-      <c r="T39" s="84">
+      <c r="P39" s="67"/>
+      <c r="Q39" s="67"/>
+      <c r="R39" s="67"/>
+      <c r="S39" s="67"/>
+      <c r="T39" s="68">
         <f t="shared" si="10"/>
         <v>3714.4933333333279</v>
       </c>
-      <c r="U39" s="84"/>
-      <c r="V39" s="84"/>
-      <c r="W39" s="85">
+      <c r="U39" s="68"/>
+      <c r="V39" s="68"/>
+      <c r="W39" s="69">
         <f t="shared" si="11"/>
         <v>3714.4933333333279</v>
       </c>
-      <c r="X39" s="85"/>
-      <c r="Y39" s="85"/>
-      <c r="Z39" s="86">
+      <c r="X39" s="69"/>
+      <c r="Y39" s="69"/>
+      <c r="Z39" s="70">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="AA39" s="86"/>
+      <c r="AA39" s="70"/>
       <c r="AB39" s="4"/>
     </row>
-    <row r="40" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="4"/>
       <c r="B40" s="7"/>
       <c r="C40" s="8"/>
@@ -6757,34 +6741,34 @@
       <c r="L40" s="8"/>
       <c r="M40" s="8"/>
       <c r="N40" s="9"/>
-      <c r="O40" s="83" t="str">
+      <c r="O40" s="67" t="str">
         <f t="shared" si="9"/>
         <v>Segurança Emive</v>
       </c>
-      <c r="P40" s="83"/>
-      <c r="Q40" s="83"/>
-      <c r="R40" s="83"/>
-      <c r="S40" s="83"/>
-      <c r="T40" s="84">
+      <c r="P40" s="67"/>
+      <c r="Q40" s="67"/>
+      <c r="R40" s="67"/>
+      <c r="S40" s="67"/>
+      <c r="T40" s="68">
         <f t="shared" si="10"/>
         <v>3072</v>
       </c>
-      <c r="U40" s="84"/>
-      <c r="V40" s="84"/>
-      <c r="W40" s="85">
+      <c r="U40" s="68"/>
+      <c r="V40" s="68"/>
+      <c r="W40" s="69">
         <f t="shared" si="11"/>
         <v>3072</v>
       </c>
-      <c r="X40" s="85"/>
-      <c r="Y40" s="85"/>
-      <c r="Z40" s="86">
+      <c r="X40" s="69"/>
+      <c r="Y40" s="69"/>
+      <c r="Z40" s="70">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="AA40" s="86"/>
+      <c r="AA40" s="70"/>
       <c r="AB40" s="4"/>
     </row>
-    <row r="41" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="4"/>
       <c r="B41" s="7"/>
       <c r="C41" s="8"/>
@@ -6799,34 +6783,34 @@
       <c r="L41" s="8"/>
       <c r="M41" s="8"/>
       <c r="N41" s="9"/>
-      <c r="O41" s="83" t="str">
+      <c r="O41" s="67" t="str">
         <f t="shared" si="9"/>
         <v>IPTU</v>
       </c>
-      <c r="P41" s="83"/>
-      <c r="Q41" s="83"/>
-      <c r="R41" s="83"/>
-      <c r="S41" s="83"/>
-      <c r="T41" s="84">
+      <c r="P41" s="67"/>
+      <c r="Q41" s="67"/>
+      <c r="R41" s="67"/>
+      <c r="S41" s="67"/>
+      <c r="T41" s="68">
         <f t="shared" si="10"/>
         <v>2569.27</v>
       </c>
-      <c r="U41" s="84"/>
-      <c r="V41" s="84"/>
-      <c r="W41" s="85">
+      <c r="U41" s="68"/>
+      <c r="V41" s="68"/>
+      <c r="W41" s="69">
         <f t="shared" si="11"/>
         <v>2569.27</v>
       </c>
-      <c r="X41" s="85"/>
-      <c r="Y41" s="85"/>
-      <c r="Z41" s="86">
+      <c r="X41" s="69"/>
+      <c r="Y41" s="69"/>
+      <c r="Z41" s="70">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="AA41" s="86"/>
+      <c r="AA41" s="70"/>
       <c r="AB41" s="4"/>
     </row>
-    <row r="42" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="4"/>
       <c r="B42" s="7"/>
       <c r="C42" s="8"/>
@@ -6841,34 +6825,34 @@
       <c r="L42" s="8"/>
       <c r="M42" s="8"/>
       <c r="N42" s="9"/>
-      <c r="O42" s="83" t="str">
+      <c r="O42" s="67" t="str">
         <f t="shared" si="9"/>
         <v>Seguro galpão</v>
       </c>
-      <c r="P42" s="83"/>
-      <c r="Q42" s="83"/>
-      <c r="R42" s="83"/>
-      <c r="S42" s="83"/>
-      <c r="T42" s="84">
+      <c r="P42" s="67"/>
+      <c r="Q42" s="67"/>
+      <c r="R42" s="67"/>
+      <c r="S42" s="67"/>
+      <c r="T42" s="68">
         <f>IF(AT15="","",AV15)</f>
         <v>2569.27</v>
       </c>
-      <c r="U42" s="84"/>
-      <c r="V42" s="84"/>
-      <c r="W42" s="85">
+      <c r="U42" s="68"/>
+      <c r="V42" s="68"/>
+      <c r="W42" s="69">
         <f t="shared" si="11"/>
         <v>2569.27</v>
       </c>
-      <c r="X42" s="85"/>
-      <c r="Y42" s="85"/>
-      <c r="Z42" s="86">
+      <c r="X42" s="69"/>
+      <c r="Y42" s="69"/>
+      <c r="Z42" s="70">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="AA42" s="86"/>
+      <c r="AA42" s="70"/>
       <c r="AB42" s="4"/>
     </row>
-    <row r="43" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="4"/>
       <c r="B43" s="7"/>
       <c r="C43" s="8"/>
@@ -6898,7 +6882,7 @@
       <c r="AA43" s="9"/>
       <c r="AB43" s="4"/>
     </row>
-    <row r="44" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="4"/>
       <c r="B44" s="7"/>
       <c r="C44" s="8"/>
@@ -6913,33 +6897,33 @@
       <c r="L44" s="8"/>
       <c r="M44" s="8"/>
       <c r="N44" s="9"/>
-      <c r="O44" s="87" t="s">
+      <c r="O44" s="63" t="s">
         <v>38</v>
       </c>
-      <c r="P44" s="87"/>
-      <c r="Q44" s="87"/>
-      <c r="R44" s="87"/>
-      <c r="S44" s="87"/>
-      <c r="T44" s="88">
+      <c r="P44" s="63"/>
+      <c r="Q44" s="63"/>
+      <c r="R44" s="63"/>
+      <c r="S44" s="63"/>
+      <c r="T44" s="64">
         <f>BC15</f>
         <v>315259.37333333329</v>
       </c>
-      <c r="U44" s="88"/>
-      <c r="V44" s="88"/>
-      <c r="W44" s="88">
+      <c r="U44" s="64"/>
+      <c r="V44" s="64"/>
+      <c r="W44" s="64">
         <f>BC6</f>
-        <v>316349.37333333329</v>
-      </c>
-      <c r="X44" s="88"/>
-      <c r="Y44" s="88"/>
-      <c r="Z44" s="89">
+        <v>319728.86333333328</v>
+      </c>
+      <c r="X44" s="64"/>
+      <c r="Y44" s="64"/>
+      <c r="Z44" s="65">
         <f>IF(OR(BC6=0,BC15=0),"",BC6/BC15-1)</f>
-        <v>3.4574705534529127E-3</v>
-      </c>
-      <c r="AA44" s="89"/>
+        <v>1.4177183544910044E-2</v>
+      </c>
+      <c r="AA44" s="65"/>
       <c r="AB44" s="4"/>
     </row>
-    <row r="45" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="4"/>
       <c r="B45" s="10"/>
       <c r="C45" s="11"/>
@@ -6969,7 +6953,7 @@
       <c r="AA45" s="12"/>
       <c r="AB45" s="4"/>
     </row>
-    <row r="46" spans="1:28" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:28" ht="6.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="4"/>
       <c r="B46" s="4"/>
       <c r="C46" s="4"/>
@@ -6999,40 +6983,40 @@
       <c r="AA46" s="4"/>
       <c r="AB46" s="4"/>
     </row>
-    <row r="47" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="4"/>
-      <c r="B47" s="90" t="str">
+      <c r="B47" s="56" t="str">
         <f>"Receitas x Despesas · "&amp;$BC$14</f>
         <v>Receitas x Despesas · Ano 2026</v>
       </c>
-      <c r="C47" s="90"/>
-      <c r="D47" s="90"/>
-      <c r="E47" s="90"/>
-      <c r="F47" s="90"/>
-      <c r="G47" s="90"/>
-      <c r="H47" s="90"/>
-      <c r="I47" s="90"/>
-      <c r="J47" s="90"/>
-      <c r="K47" s="90"/>
-      <c r="L47" s="90"/>
-      <c r="M47" s="90"/>
-      <c r="N47" s="90"/>
-      <c r="O47" s="90"/>
-      <c r="P47" s="90"/>
-      <c r="Q47" s="90"/>
-      <c r="R47" s="90"/>
-      <c r="S47" s="90"/>
-      <c r="T47" s="90"/>
-      <c r="U47" s="90"/>
-      <c r="V47" s="90"/>
-      <c r="W47" s="90"/>
-      <c r="X47" s="90"/>
-      <c r="Y47" s="90"/>
-      <c r="Z47" s="90"/>
-      <c r="AA47" s="90"/>
+      <c r="C47" s="56"/>
+      <c r="D47" s="56"/>
+      <c r="E47" s="56"/>
+      <c r="F47" s="56"/>
+      <c r="G47" s="56"/>
+      <c r="H47" s="56"/>
+      <c r="I47" s="56"/>
+      <c r="J47" s="56"/>
+      <c r="K47" s="56"/>
+      <c r="L47" s="56"/>
+      <c r="M47" s="56"/>
+      <c r="N47" s="56"/>
+      <c r="O47" s="56"/>
+      <c r="P47" s="56"/>
+      <c r="Q47" s="56"/>
+      <c r="R47" s="56"/>
+      <c r="S47" s="56"/>
+      <c r="T47" s="56"/>
+      <c r="U47" s="56"/>
+      <c r="V47" s="56"/>
+      <c r="W47" s="56"/>
+      <c r="X47" s="56"/>
+      <c r="Y47" s="56"/>
+      <c r="Z47" s="56"/>
+      <c r="AA47" s="56"/>
       <c r="AB47" s="4"/>
     </row>
-    <row r="48" spans="1:28" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:28" ht="6.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="4"/>
       <c r="B48" s="4"/>
       <c r="C48" s="4"/>
@@ -7062,187 +7046,187 @@
       <c r="AA48" s="4"/>
       <c r="AB48" s="4"/>
     </row>
-    <row r="49" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="4"/>
-      <c r="B49" s="91" t="s">
+      <c r="B49" s="66" t="s">
         <v>39</v>
       </c>
-      <c r="C49" s="91"/>
-      <c r="D49" s="91"/>
-      <c r="E49" s="91"/>
-      <c r="F49" s="91" t="s">
+      <c r="C49" s="66"/>
+      <c r="D49" s="66"/>
+      <c r="E49" s="66"/>
+      <c r="F49" s="66" t="s">
         <v>40</v>
       </c>
-      <c r="G49" s="91"/>
-      <c r="H49" s="91"/>
-      <c r="I49" s="91"/>
-      <c r="J49" s="91" t="s">
+      <c r="G49" s="66"/>
+      <c r="H49" s="66"/>
+      <c r="I49" s="66"/>
+      <c r="J49" s="66" t="s">
         <v>41</v>
       </c>
-      <c r="K49" s="91"/>
-      <c r="L49" s="91"/>
-      <c r="M49" s="91"/>
-      <c r="N49" s="91" t="s">
+      <c r="K49" s="66"/>
+      <c r="L49" s="66"/>
+      <c r="M49" s="66"/>
+      <c r="N49" s="66" t="s">
         <v>42</v>
       </c>
-      <c r="O49" s="91"/>
-      <c r="P49" s="91"/>
-      <c r="Q49" s="91"/>
-      <c r="R49" s="91" t="s">
+      <c r="O49" s="66"/>
+      <c r="P49" s="66"/>
+      <c r="Q49" s="66"/>
+      <c r="R49" s="66" t="s">
         <v>43</v>
       </c>
-      <c r="S49" s="91"/>
-      <c r="T49" s="91"/>
-      <c r="U49" s="91"/>
-      <c r="V49" s="91"/>
-      <c r="W49" s="91" t="s">
+      <c r="S49" s="66"/>
+      <c r="T49" s="66"/>
+      <c r="U49" s="66"/>
+      <c r="V49" s="66"/>
+      <c r="W49" s="66" t="s">
         <v>44</v>
       </c>
-      <c r="X49" s="91"/>
-      <c r="Y49" s="91"/>
-      <c r="Z49" s="91"/>
-      <c r="AA49" s="91"/>
+      <c r="X49" s="66"/>
+      <c r="Y49" s="66"/>
+      <c r="Z49" s="66"/>
+      <c r="AA49" s="66"/>
       <c r="AB49" s="52"/>
     </row>
-    <row r="50" spans="1:28" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:28" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="4"/>
-      <c r="B50" s="92">
+      <c r="B50" s="57">
         <f>BC17</f>
         <v>0</v>
       </c>
-      <c r="C50" s="92"/>
-      <c r="D50" s="92"/>
-      <c r="E50" s="92"/>
-      <c r="F50" s="92">
+      <c r="C50" s="57"/>
+      <c r="D50" s="57"/>
+      <c r="E50" s="57"/>
+      <c r="F50" s="57">
         <f>BC6</f>
-        <v>316349.37333333329</v>
-      </c>
-      <c r="G50" s="92"/>
-      <c r="H50" s="92"/>
-      <c r="I50" s="92"/>
-      <c r="J50" s="92">
+        <v>319728.86333333328</v>
+      </c>
+      <c r="G50" s="57"/>
+      <c r="H50" s="57"/>
+      <c r="I50" s="57"/>
+      <c r="J50" s="57">
         <f>BC17-BC6</f>
-        <v>-316349.37333333329</v>
-      </c>
-      <c r="K50" s="92"/>
-      <c r="L50" s="92"/>
-      <c r="M50" s="92"/>
-      <c r="N50" s="93">
+        <v>-319728.86333333328</v>
+      </c>
+      <c r="K50" s="57"/>
+      <c r="L50" s="57"/>
+      <c r="M50" s="57"/>
+      <c r="N50" s="58">
         <f>IF(BC17=0,0,(BC17-BC6)/BC17)</f>
         <v>0</v>
       </c>
-      <c r="O50" s="93"/>
-      <c r="P50" s="93"/>
-      <c r="Q50" s="93"/>
-      <c r="R50" s="92">
+      <c r="O50" s="58"/>
+      <c r="P50" s="58"/>
+      <c r="Q50" s="58"/>
+      <c r="R50" s="57">
         <f>IF(BC19=0,0,BC18/BC19)</f>
         <v>0</v>
       </c>
-      <c r="S50" s="92"/>
-      <c r="T50" s="92"/>
-      <c r="U50" s="92"/>
-      <c r="V50" s="92"/>
-      <c r="W50" s="92">
+      <c r="S50" s="57"/>
+      <c r="T50" s="57"/>
+      <c r="U50" s="57"/>
+      <c r="V50" s="57"/>
+      <c r="W50" s="57">
         <f>BC20/12</f>
-        <v>26362.447777777776</v>
-      </c>
-      <c r="X50" s="92"/>
-      <c r="Y50" s="92"/>
-      <c r="Z50" s="92"/>
-      <c r="AA50" s="92"/>
+        <v>26644.07194444444</v>
+      </c>
+      <c r="X50" s="57"/>
+      <c r="Y50" s="57"/>
+      <c r="Z50" s="57"/>
+      <c r="AA50" s="57"/>
       <c r="AB50" s="52"/>
     </row>
-    <row r="51" spans="1:28" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:28" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="4"/>
-      <c r="B51" s="92"/>
-      <c r="C51" s="92"/>
-      <c r="D51" s="92"/>
-      <c r="E51" s="92"/>
-      <c r="F51" s="92"/>
-      <c r="G51" s="92"/>
-      <c r="H51" s="92"/>
-      <c r="I51" s="92"/>
-      <c r="J51" s="92"/>
-      <c r="K51" s="92"/>
-      <c r="L51" s="92"/>
-      <c r="M51" s="92"/>
-      <c r="N51" s="93"/>
-      <c r="O51" s="93"/>
-      <c r="P51" s="93"/>
-      <c r="Q51" s="93"/>
-      <c r="R51" s="92"/>
-      <c r="S51" s="92"/>
-      <c r="T51" s="92"/>
-      <c r="U51" s="92"/>
-      <c r="V51" s="92"/>
-      <c r="W51" s="92"/>
-      <c r="X51" s="92"/>
-      <c r="Y51" s="92"/>
-      <c r="Z51" s="92"/>
-      <c r="AA51" s="92"/>
+      <c r="B51" s="57"/>
+      <c r="C51" s="57"/>
+      <c r="D51" s="57"/>
+      <c r="E51" s="57"/>
+      <c r="F51" s="57"/>
+      <c r="G51" s="57"/>
+      <c r="H51" s="57"/>
+      <c r="I51" s="57"/>
+      <c r="J51" s="57"/>
+      <c r="K51" s="57"/>
+      <c r="L51" s="57"/>
+      <c r="M51" s="57"/>
+      <c r="N51" s="58"/>
+      <c r="O51" s="58"/>
+      <c r="P51" s="58"/>
+      <c r="Q51" s="58"/>
+      <c r="R51" s="57"/>
+      <c r="S51" s="57"/>
+      <c r="T51" s="57"/>
+      <c r="U51" s="57"/>
+      <c r="V51" s="57"/>
+      <c r="W51" s="57"/>
+      <c r="X51" s="57"/>
+      <c r="Y51" s="57"/>
+      <c r="Z51" s="57"/>
+      <c r="AA51" s="57"/>
       <c r="AB51" s="52"/>
     </row>
-    <row r="52" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="4"/>
-      <c r="B52" s="94" t="s">
+      <c r="B52" s="59" t="s">
         <v>45</v>
       </c>
-      <c r="C52" s="94"/>
-      <c r="D52" s="95">
+      <c r="C52" s="59"/>
+      <c r="D52" s="60">
         <f>BC18</f>
         <v>0</v>
       </c>
-      <c r="E52" s="95"/>
-      <c r="F52" s="94" t="s">
+      <c r="E52" s="60"/>
+      <c r="F52" s="59" t="s">
         <v>7</v>
       </c>
-      <c r="G52" s="94"/>
-      <c r="H52" s="95">
+      <c r="G52" s="59"/>
+      <c r="H52" s="60">
         <f>BC7</f>
         <v>315259.37333333329</v>
       </c>
-      <c r="I52" s="95"/>
-      <c r="J52" s="94" t="s">
+      <c r="I52" s="60"/>
+      <c r="J52" s="59" t="s">
         <v>46</v>
       </c>
-      <c r="K52" s="94"/>
-      <c r="L52" s="96">
+      <c r="K52" s="59"/>
+      <c r="L52" s="61">
         <f>IF(BC17=0,0,(BC17-BC6)/BC17)</f>
         <v>0</v>
       </c>
-      <c r="M52" s="96"/>
-      <c r="N52" s="94" t="s">
+      <c r="M52" s="61"/>
+      <c r="N52" s="59" t="s">
         <v>13</v>
       </c>
-      <c r="O52" s="94"/>
-      <c r="P52" s="95">
+      <c r="O52" s="59"/>
+      <c r="P52" s="60">
         <f>BC17-BC6</f>
-        <v>-316349.37333333329</v>
-      </c>
-      <c r="Q52" s="95"/>
-      <c r="R52" s="94" t="s">
+        <v>-319728.86333333328</v>
+      </c>
+      <c r="Q52" s="60"/>
+      <c r="R52" s="59" t="s">
         <v>47</v>
       </c>
-      <c r="S52" s="94"/>
-      <c r="T52" s="97">
+      <c r="S52" s="59"/>
+      <c r="T52" s="62">
         <f>BC19</f>
         <v>0</v>
       </c>
-      <c r="U52" s="97"/>
-      <c r="V52" s="97"/>
-      <c r="W52" s="94" t="s">
+      <c r="U52" s="62"/>
+      <c r="V52" s="62"/>
+      <c r="W52" s="59" t="s">
         <v>48</v>
       </c>
-      <c r="X52" s="94"/>
-      <c r="Y52" s="95">
+      <c r="X52" s="59"/>
+      <c r="Y52" s="60">
         <f>BC20</f>
-        <v>316349.37333333329</v>
-      </c>
-      <c r="Z52" s="95"/>
-      <c r="AA52" s="95"/>
+        <v>319728.86333333328</v>
+      </c>
+      <c r="Z52" s="60"/>
+      <c r="AA52" s="60"/>
       <c r="AB52" s="52"/>
     </row>
-    <row r="53" spans="1:28" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:28" ht="6.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="4"/>
       <c r="B53" s="4"/>
       <c r="C53" s="4"/>
@@ -7272,39 +7256,39 @@
       <c r="AA53" s="4"/>
       <c r="AB53" s="52"/>
     </row>
-    <row r="54" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="4"/>
-      <c r="B54" s="90" t="s">
+      <c r="B54" s="56" t="s">
         <v>49</v>
       </c>
-      <c r="C54" s="90"/>
-      <c r="D54" s="90"/>
-      <c r="E54" s="90"/>
-      <c r="F54" s="90"/>
-      <c r="G54" s="90"/>
-      <c r="H54" s="90"/>
-      <c r="I54" s="90"/>
-      <c r="J54" s="90"/>
-      <c r="K54" s="90"/>
-      <c r="L54" s="90"/>
-      <c r="M54" s="90"/>
-      <c r="N54" s="90"/>
-      <c r="O54" s="90"/>
-      <c r="P54" s="90"/>
-      <c r="Q54" s="90"/>
-      <c r="R54" s="90"/>
-      <c r="S54" s="90"/>
-      <c r="T54" s="90"/>
-      <c r="U54" s="90"/>
-      <c r="V54" s="90"/>
-      <c r="W54" s="90"/>
-      <c r="X54" s="90"/>
-      <c r="Y54" s="90"/>
-      <c r="Z54" s="90"/>
-      <c r="AA54" s="90"/>
+      <c r="C54" s="56"/>
+      <c r="D54" s="56"/>
+      <c r="E54" s="56"/>
+      <c r="F54" s="56"/>
+      <c r="G54" s="56"/>
+      <c r="H54" s="56"/>
+      <c r="I54" s="56"/>
+      <c r="J54" s="56"/>
+      <c r="K54" s="56"/>
+      <c r="L54" s="56"/>
+      <c r="M54" s="56"/>
+      <c r="N54" s="56"/>
+      <c r="O54" s="56"/>
+      <c r="P54" s="56"/>
+      <c r="Q54" s="56"/>
+      <c r="R54" s="56"/>
+      <c r="S54" s="56"/>
+      <c r="T54" s="56"/>
+      <c r="U54" s="56"/>
+      <c r="V54" s="56"/>
+      <c r="W54" s="56"/>
+      <c r="X54" s="56"/>
+      <c r="Y54" s="56"/>
+      <c r="Z54" s="56"/>
+      <c r="AA54" s="56"/>
       <c r="AB54" s="52"/>
     </row>
-    <row r="55" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="4"/>
       <c r="B55" s="8"/>
       <c r="C55" s="8"/>
@@ -7334,7 +7318,7 @@
       <c r="AA55" s="8"/>
       <c r="AB55" s="52"/>
     </row>
-    <row r="56" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="4"/>
       <c r="B56" s="8"/>
       <c r="C56" s="8"/>
@@ -7364,7 +7348,7 @@
       <c r="AA56" s="8"/>
       <c r="AB56" s="52"/>
     </row>
-    <row r="57" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="4"/>
       <c r="B57" s="8"/>
       <c r="C57" s="8"/>
@@ -7394,7 +7378,7 @@
       <c r="AA57" s="8"/>
       <c r="AB57" s="52"/>
     </row>
-    <row r="58" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="4"/>
       <c r="B58" s="8"/>
       <c r="C58" s="8"/>
@@ -7424,7 +7408,7 @@
       <c r="AA58" s="8"/>
       <c r="AB58" s="52"/>
     </row>
-    <row r="59" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A59" s="4"/>
       <c r="B59" s="8"/>
       <c r="C59" s="8"/>
@@ -7454,7 +7438,7 @@
       <c r="AA59" s="8"/>
       <c r="AB59" s="52"/>
     </row>
-    <row r="60" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="4"/>
       <c r="B60" s="8"/>
       <c r="C60" s="8"/>
@@ -7484,7 +7468,7 @@
       <c r="AA60" s="8"/>
       <c r="AB60" s="52"/>
     </row>
-    <row r="61" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A61" s="4"/>
       <c r="B61" s="8"/>
       <c r="C61" s="8"/>
@@ -7514,7 +7498,7 @@
       <c r="AA61" s="8"/>
       <c r="AB61" s="52"/>
     </row>
-    <row r="62" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" s="4"/>
       <c r="B62" s="8"/>
       <c r="C62" s="8"/>
@@ -7544,7 +7528,7 @@
       <c r="AA62" s="8"/>
       <c r="AB62" s="52"/>
     </row>
-    <row r="63" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A63" s="4"/>
       <c r="B63" s="8"/>
       <c r="C63" s="8"/>
@@ -7574,7 +7558,7 @@
       <c r="AA63" s="8"/>
       <c r="AB63" s="52"/>
     </row>
-    <row r="64" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A64" s="4"/>
       <c r="B64" s="8"/>
       <c r="C64" s="8"/>
@@ -7604,7 +7588,7 @@
       <c r="AA64" s="8"/>
       <c r="AB64" s="52"/>
     </row>
-    <row r="65" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A65" s="4"/>
       <c r="B65" s="8"/>
       <c r="C65" s="8"/>
@@ -7634,7 +7618,7 @@
       <c r="AA65" s="8"/>
       <c r="AB65" s="52"/>
     </row>
-    <row r="66" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" s="4"/>
       <c r="B66" s="8"/>
       <c r="C66" s="8"/>
@@ -7664,7 +7648,7 @@
       <c r="AA66" s="8"/>
       <c r="AB66" s="52"/>
     </row>
-    <row r="67" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A67" s="4"/>
       <c r="B67" s="8"/>
       <c r="C67" s="8"/>
@@ -7694,7 +7678,7 @@
       <c r="AA67" s="8"/>
       <c r="AB67" s="52"/>
     </row>
-    <row r="68" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A68" s="4"/>
       <c r="B68" s="8"/>
       <c r="C68" s="8"/>
@@ -7724,7 +7708,7 @@
       <c r="AA68" s="8"/>
       <c r="AB68" s="52"/>
     </row>
-    <row r="69" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A69" s="4"/>
       <c r="B69" s="8"/>
       <c r="C69" s="8"/>
@@ -7756,6 +7740,113 @@
     </row>
   </sheetData>
   <mergeCells count="126">
+    <mergeCell ref="B1:AA1"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="G3:K3"/>
+    <mergeCell ref="L3:Q3"/>
+    <mergeCell ref="R3:T4"/>
+    <mergeCell ref="U3:W4"/>
+    <mergeCell ref="X3:Y4"/>
+    <mergeCell ref="Z3:AA4"/>
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="G4:K4"/>
+    <mergeCell ref="L4:Q4"/>
+    <mergeCell ref="T6:U6"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="X6:Y6"/>
+    <mergeCell ref="Z6:AA6"/>
+    <mergeCell ref="B8:E8"/>
+    <mergeCell ref="F8:I8"/>
+    <mergeCell ref="J8:M8"/>
+    <mergeCell ref="N8:Q8"/>
+    <mergeCell ref="R8:V8"/>
+    <mergeCell ref="W8:AA8"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="F6:G6"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="L6:M6"/>
+    <mergeCell ref="N6:O6"/>
+    <mergeCell ref="P6:Q6"/>
+    <mergeCell ref="R6:S6"/>
+    <mergeCell ref="B9:E10"/>
+    <mergeCell ref="F9:I10"/>
+    <mergeCell ref="J9:M10"/>
+    <mergeCell ref="N9:Q10"/>
+    <mergeCell ref="R9:V10"/>
+    <mergeCell ref="W9:AA10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="H11:I11"/>
+    <mergeCell ref="J11:K11"/>
+    <mergeCell ref="L11:M11"/>
+    <mergeCell ref="N11:O11"/>
+    <mergeCell ref="P11:Q11"/>
+    <mergeCell ref="R11:S11"/>
+    <mergeCell ref="T11:V11"/>
+    <mergeCell ref="W11:X11"/>
+    <mergeCell ref="Y11:AA11"/>
+    <mergeCell ref="B13:Q13"/>
+    <mergeCell ref="R13:AA13"/>
+    <mergeCell ref="B30:N30"/>
+    <mergeCell ref="O30:AA30"/>
+    <mergeCell ref="O32:S32"/>
+    <mergeCell ref="T32:V32"/>
+    <mergeCell ref="W32:Y32"/>
+    <mergeCell ref="Z32:AA32"/>
+    <mergeCell ref="O33:S33"/>
+    <mergeCell ref="T33:V33"/>
+    <mergeCell ref="W33:Y33"/>
+    <mergeCell ref="Z33:AA33"/>
+    <mergeCell ref="O34:S34"/>
+    <mergeCell ref="T34:V34"/>
+    <mergeCell ref="W34:Y34"/>
+    <mergeCell ref="Z34:AA34"/>
+    <mergeCell ref="O35:S35"/>
+    <mergeCell ref="T35:V35"/>
+    <mergeCell ref="W35:Y35"/>
+    <mergeCell ref="Z35:AA35"/>
+    <mergeCell ref="O36:S36"/>
+    <mergeCell ref="T36:V36"/>
+    <mergeCell ref="W36:Y36"/>
+    <mergeCell ref="Z36:AA36"/>
+    <mergeCell ref="O37:S37"/>
+    <mergeCell ref="T37:V37"/>
+    <mergeCell ref="W37:Y37"/>
+    <mergeCell ref="Z37:AA37"/>
+    <mergeCell ref="O38:S38"/>
+    <mergeCell ref="T38:V38"/>
+    <mergeCell ref="W38:Y38"/>
+    <mergeCell ref="Z38:AA38"/>
+    <mergeCell ref="O39:S39"/>
+    <mergeCell ref="T39:V39"/>
+    <mergeCell ref="W39:Y39"/>
+    <mergeCell ref="Z39:AA39"/>
+    <mergeCell ref="O40:S40"/>
+    <mergeCell ref="T40:V40"/>
+    <mergeCell ref="W40:Y40"/>
+    <mergeCell ref="Z40:AA40"/>
+    <mergeCell ref="O41:S41"/>
+    <mergeCell ref="T41:V41"/>
+    <mergeCell ref="W41:Y41"/>
+    <mergeCell ref="Z41:AA41"/>
+    <mergeCell ref="O42:S42"/>
+    <mergeCell ref="T42:V42"/>
+    <mergeCell ref="W42:Y42"/>
+    <mergeCell ref="Z42:AA42"/>
+    <mergeCell ref="O44:S44"/>
+    <mergeCell ref="T44:V44"/>
+    <mergeCell ref="W44:Y44"/>
+    <mergeCell ref="Z44:AA44"/>
+    <mergeCell ref="B47:AA47"/>
+    <mergeCell ref="B49:E49"/>
+    <mergeCell ref="F49:I49"/>
+    <mergeCell ref="J49:M49"/>
+    <mergeCell ref="N49:Q49"/>
+    <mergeCell ref="R49:V49"/>
+    <mergeCell ref="W49:AA49"/>
     <mergeCell ref="B54:AA54"/>
     <mergeCell ref="B50:E51"/>
     <mergeCell ref="F50:I51"/>
@@ -7775,113 +7866,6 @@
     <mergeCell ref="T52:V52"/>
     <mergeCell ref="W52:X52"/>
     <mergeCell ref="Y52:AA52"/>
-    <mergeCell ref="O44:S44"/>
-    <mergeCell ref="T44:V44"/>
-    <mergeCell ref="W44:Y44"/>
-    <mergeCell ref="Z44:AA44"/>
-    <mergeCell ref="B47:AA47"/>
-    <mergeCell ref="B49:E49"/>
-    <mergeCell ref="F49:I49"/>
-    <mergeCell ref="J49:M49"/>
-    <mergeCell ref="N49:Q49"/>
-    <mergeCell ref="R49:V49"/>
-    <mergeCell ref="W49:AA49"/>
-    <mergeCell ref="O40:S40"/>
-    <mergeCell ref="T40:V40"/>
-    <mergeCell ref="W40:Y40"/>
-    <mergeCell ref="Z40:AA40"/>
-    <mergeCell ref="O41:S41"/>
-    <mergeCell ref="T41:V41"/>
-    <mergeCell ref="W41:Y41"/>
-    <mergeCell ref="Z41:AA41"/>
-    <mergeCell ref="O42:S42"/>
-    <mergeCell ref="T42:V42"/>
-    <mergeCell ref="W42:Y42"/>
-    <mergeCell ref="Z42:AA42"/>
-    <mergeCell ref="O37:S37"/>
-    <mergeCell ref="T37:V37"/>
-    <mergeCell ref="W37:Y37"/>
-    <mergeCell ref="Z37:AA37"/>
-    <mergeCell ref="O38:S38"/>
-    <mergeCell ref="T38:V38"/>
-    <mergeCell ref="W38:Y38"/>
-    <mergeCell ref="Z38:AA38"/>
-    <mergeCell ref="O39:S39"/>
-    <mergeCell ref="T39:V39"/>
-    <mergeCell ref="W39:Y39"/>
-    <mergeCell ref="Z39:AA39"/>
-    <mergeCell ref="O34:S34"/>
-    <mergeCell ref="T34:V34"/>
-    <mergeCell ref="W34:Y34"/>
-    <mergeCell ref="Z34:AA34"/>
-    <mergeCell ref="O35:S35"/>
-    <mergeCell ref="T35:V35"/>
-    <mergeCell ref="W35:Y35"/>
-    <mergeCell ref="Z35:AA35"/>
-    <mergeCell ref="O36:S36"/>
-    <mergeCell ref="T36:V36"/>
-    <mergeCell ref="W36:Y36"/>
-    <mergeCell ref="Z36:AA36"/>
-    <mergeCell ref="B13:Q13"/>
-    <mergeCell ref="R13:AA13"/>
-    <mergeCell ref="B30:N30"/>
-    <mergeCell ref="O30:AA30"/>
-    <mergeCell ref="O32:S32"/>
-    <mergeCell ref="T32:V32"/>
-    <mergeCell ref="W32:Y32"/>
-    <mergeCell ref="Z32:AA32"/>
-    <mergeCell ref="O33:S33"/>
-    <mergeCell ref="T33:V33"/>
-    <mergeCell ref="W33:Y33"/>
-    <mergeCell ref="Z33:AA33"/>
-    <mergeCell ref="B9:E10"/>
-    <mergeCell ref="F9:I10"/>
-    <mergeCell ref="J9:M10"/>
-    <mergeCell ref="N9:Q10"/>
-    <mergeCell ref="R9:V10"/>
-    <mergeCell ref="W9:AA10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="H11:I11"/>
-    <mergeCell ref="J11:K11"/>
-    <mergeCell ref="L11:M11"/>
-    <mergeCell ref="N11:O11"/>
-    <mergeCell ref="P11:Q11"/>
-    <mergeCell ref="R11:S11"/>
-    <mergeCell ref="T11:V11"/>
-    <mergeCell ref="W11:X11"/>
-    <mergeCell ref="Y11:AA11"/>
-    <mergeCell ref="T6:U6"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="X6:Y6"/>
-    <mergeCell ref="Z6:AA6"/>
-    <mergeCell ref="B8:E8"/>
-    <mergeCell ref="F8:I8"/>
-    <mergeCell ref="J8:M8"/>
-    <mergeCell ref="N8:Q8"/>
-    <mergeCell ref="R8:V8"/>
-    <mergeCell ref="W8:AA8"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="F6:G6"/>
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="L6:M6"/>
-    <mergeCell ref="N6:O6"/>
-    <mergeCell ref="P6:Q6"/>
-    <mergeCell ref="R6:S6"/>
-    <mergeCell ref="B1:AA1"/>
-    <mergeCell ref="B3:F3"/>
-    <mergeCell ref="G3:K3"/>
-    <mergeCell ref="L3:Q3"/>
-    <mergeCell ref="R3:T4"/>
-    <mergeCell ref="U3:W4"/>
-    <mergeCell ref="X3:Y4"/>
-    <mergeCell ref="Z3:AA4"/>
-    <mergeCell ref="B4:F4"/>
-    <mergeCell ref="G4:K4"/>
-    <mergeCell ref="L4:Q4"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:AA6">
     <cfRule type="expression" dxfId="17" priority="2">
@@ -7957,7 +7941,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" sqref="U3">
+    <dataValidation type="list" sqref="U3" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Ano,Jan,Fev,Mar,Abr,Mai,Jun,Jul,Ago,Set,Out,Nov,Dez"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -7987,32 +7971,32 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <tabColor rgb="FFFFC000"/>
   </sheetPr>
   <dimension ref="A1:P25"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="58.5703125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="55.140625" style="1" customWidth="1"/>
-    <col min="3" max="4" width="12.42578125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="12.7109375" style="1" customWidth="1"/>
-    <col min="6" max="14" width="12.42578125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="58.5546875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="55.109375" style="1" customWidth="1"/>
+    <col min="3" max="4" width="12.44140625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="12.6640625" style="1" customWidth="1"/>
+    <col min="6" max="14" width="12.44140625" style="1" customWidth="1"/>
     <col min="15" max="16" width="15" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="13" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="54" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="3" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="15" t="s">
         <v>52</v>
       </c>
@@ -8053,7 +8037,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="17" t="s">
         <v>12</v>
       </c>
@@ -8103,7 +8087,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="5" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="18" t="str">
         <f>IF(Cadastro!B5="","",Cadastro!B5)</f>
         <v>Água</v>
@@ -8157,7 +8141,7 @@
         <v>93.19</v>
       </c>
     </row>
-    <row r="6" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="18" t="str">
         <f>IF(Cadastro!B6="","",Cadastro!B6)</f>
         <v>Energia</v>
@@ -8211,7 +8195,7 @@
         <v>145.19000000000003</v>
       </c>
     </row>
-    <row r="7" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="18" t="str">
         <f>IF(Cadastro!B7="","",Cadastro!B7)</f>
         <v>Seguro galpão</v>
@@ -8261,7 +8245,7 @@
         <v>367.0385714285714</v>
       </c>
     </row>
-    <row r="8" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="18" t="str">
         <f>IF(Cadastro!B8="","",Cadastro!B8)</f>
         <v>Segurança Emive</v>
@@ -8315,7 +8299,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="9" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="18" t="str">
         <f>IF(Cadastro!B9="","",Cadastro!B9)</f>
         <v>Dedetização</v>
@@ -8369,7 +8353,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="10" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="18" t="str">
         <f>IF(Cadastro!B10="","",Cadastro!B10)</f>
         <v>IPTU</v>
@@ -8423,7 +8407,7 @@
         <v>321.15875</v>
       </c>
     </row>
-    <row r="11" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="18" t="str">
         <f>IF(Cadastro!B11="","",Cadastro!B11)</f>
         <v>Controle de Ponto</v>
@@ -8477,7 +8461,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="12" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="18" t="str">
         <f>IF(Cadastro!B12="","",Cadastro!B12)</f>
         <v>Extintores</v>
@@ -8531,7 +8515,7 @@
         <v>71.25</v>
       </c>
     </row>
-    <row r="13" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="18" t="str">
         <f>IF(Cadastro!B13="","",Cadastro!B13)</f>
         <v>Internet</v>
@@ -8585,7 +8569,7 @@
         <v>167.71</v>
       </c>
     </row>
-    <row r="14" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="18" t="str">
         <f>IF(Cadastro!B14="","",Cadastro!B14)</f>
         <v>Funcionários</v>
@@ -8639,7 +8623,7 @@
         <v>14212.81</v>
       </c>
     </row>
-    <row r="15" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="18" t="s">
         <v>101</v>
       </c>
@@ -8687,7 +8671,7 @@
         <v>3841.6275000000001</v>
       </c>
     </row>
-    <row r="16" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="55" t="s">
         <v>110</v>
       </c>
@@ -8724,7 +8708,7 @@
         <v>2655.75</v>
       </c>
     </row>
-    <row r="17" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="18" t="str">
         <f>IF(Cadastro!B17="","",Cadastro!B17)</f>
         <v>Tubete</v>
@@ -8770,7 +8754,7 @@
         <v>14035.15</v>
       </c>
     </row>
-    <row r="18" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="18" t="str">
         <f>IF(Cadastro!B18="","",Cadastro!B18)</f>
         <v>Manutenção Predial</v>
@@ -8814,7 +8798,7 @@
         <v>599.71428571428567</v>
       </c>
     </row>
-    <row r="19" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="18" t="str">
         <f>IF(Cadastro!B19="","",Cadastro!B19)</f>
         <v>Seguro do Caminhão</v>
@@ -8860,7 +8844,7 @@
         <v>464.31166666666599</v>
       </c>
     </row>
-    <row r="20" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="55" t="str">
         <f>IF(Cadastro!B20="","",Cadastro!B20)</f>
         <v>Parcela Caminhão</v>
@@ -8893,20 +8877,22 @@
       <c r="J20" s="20">
         <v>3379.49</v>
       </c>
-      <c r="K20" s="20"/>
+      <c r="K20" s="20">
+        <v>3379.49</v>
+      </c>
       <c r="L20" s="20"/>
       <c r="M20" s="20"/>
       <c r="N20" s="20"/>
       <c r="O20" s="21">
         <f t="shared" si="0"/>
-        <v>27035.919999999991</v>
+        <v>30415.409999999989</v>
       </c>
       <c r="P20" s="22">
         <f t="shared" si="1"/>
         <v>3379.4899999999989</v>
       </c>
     </row>
-    <row r="21" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="55" t="str">
         <f>IF(Cadastro!B21="","",Cadastro!B21)</f>
         <v>Despesas Pessoal (EPI, Farda e Ferramentas, Diaristas)</v>
@@ -8939,7 +8925,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="22" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="18" t="str">
         <f>IF(Cadastro!B22="","",Cadastro!B22)</f>
         <v xml:space="preserve">Outras Despesas </v>
@@ -8984,7 +8970,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="24" t="s">
         <v>55</v>
       </c>
@@ -9023,7 +9009,7 @@
       </c>
       <c r="K23" s="24">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>3379.49</v>
       </c>
       <c r="L23" s="24">
         <f t="shared" si="2"/>
@@ -9039,14 +9025,14 @@
       </c>
       <c r="O23" s="24">
         <f t="shared" si="2"/>
-        <v>316349.37333333329</v>
+        <v>319728.86333333328</v>
       </c>
       <c r="P23" s="24">
         <f t="shared" si="2"/>
         <v>41175.390773809522</v>
       </c>
     </row>
-    <row r="24" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="25" t="s">
         <v>56</v>
       </c>
@@ -9085,7 +9071,7 @@
       </c>
       <c r="K24" s="27">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L24" s="27">
         <f t="shared" si="3"/>
@@ -9100,7 +9086,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="25" t="s">
         <v>57</v>
       </c>
@@ -9139,7 +9125,7 @@
       </c>
       <c r="K25" s="28" t="str">
         <f>IF(K24=0,"Pendente",IF(K24&lt;COUNTA(Cadastro!$B$5:$B$22),"Parcial","Completo"))</f>
-        <v>Pendente</v>
+        <v>Parcial</v>
       </c>
       <c r="L25" s="28" t="str">
         <f>IF(L24=0,"Pendente",IF(L24&lt;COUNTA(Cadastro!$B$5:$B$22),"Parcial","Completo"))</f>
@@ -9167,7 +9153,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" errorTitle="Valor inválido" error="Digite apenas números (valor em R$)." sqref="C5:N15 K16:N16 C17:N22">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" errorTitle="Valor inválido" error="Digite apenas números (valor em R$)." sqref="C5:N15 K16:N16 C17:N22" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>0</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -9178,12 +9164,12 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <tabColor rgb="FF70AD47"/>
   </sheetPr>
   <dimension ref="A1:P17"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="26" style="1" customWidth="1"/>
     <col min="2" max="2" width="20" style="1" customWidth="1"/>
@@ -9191,17 +9177,17 @@
     <col min="15" max="16" width="14" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="29" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="30" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="3" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="31" t="s">
         <v>52</v>
       </c>
@@ -9242,7 +9228,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="33" t="s">
         <v>11</v>
       </c>
@@ -9292,7 +9278,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="5" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="34" t="s">
         <v>61</v>
       </c>
@@ -9320,7 +9306,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="34"/>
       <c r="B6" s="34"/>
       <c r="C6" s="36"/>
@@ -9344,7 +9330,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="34"/>
       <c r="B7" s="34"/>
       <c r="C7" s="36"/>
@@ -9368,7 +9354,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="34"/>
       <c r="B8" s="34"/>
       <c r="C8" s="36"/>
@@ -9392,7 +9378,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="34"/>
       <c r="B9" s="34"/>
       <c r="C9" s="36"/>
@@ -9416,7 +9402,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="34"/>
       <c r="B10" s="34"/>
       <c r="C10" s="36"/>
@@ -9440,7 +9426,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="34"/>
       <c r="B11" s="34"/>
       <c r="C11" s="36"/>
@@ -9464,7 +9450,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="34"/>
       <c r="B12" s="34"/>
       <c r="C12" s="36"/>
@@ -9488,7 +9474,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="34"/>
       <c r="B13" s="34"/>
       <c r="C13" s="36"/>
@@ -9512,7 +9498,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="34"/>
       <c r="B14" s="34"/>
       <c r="C14" s="36"/>
@@ -9536,7 +9522,7 @@
         <v/>
       </c>
     </row>
-    <row r="16" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="38" t="s">
         <v>55</v>
       </c>
@@ -9598,7 +9584,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="17" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="41" t="s">
         <v>63</v>
       </c>
@@ -9654,7 +9640,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" errorTitle="Valor inválido" error="Digite apenas números (valor em R$)." sqref="C5:N14">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" errorTitle="Valor inválido" error="Digite apenas números (valor em R$)." sqref="C5:N14" xr:uid="{00000000-0002-0000-0200-000000000000}">
       <formula1>0</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -9665,30 +9651,30 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
     <tabColor rgb="FFA6A6A6"/>
   </sheetPr>
   <dimension ref="A1:P23"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="77" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18" style="1" customWidth="1"/>
-    <col min="3" max="14" width="12.42578125" style="1" customWidth="1"/>
+    <col min="3" max="14" width="12.44140625" style="1" customWidth="1"/>
     <col min="15" max="16" width="15" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="13" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="14" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="3" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="15" t="s">
         <v>52</v>
       </c>
@@ -9729,7 +9715,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="17" t="s">
         <v>12</v>
       </c>
@@ -9779,7 +9765,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="5" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="18" t="str">
         <f>IF(Cadastro!B5="","",Cadastro!B5)</f>
         <v>Água</v>
@@ -9833,7 +9819,7 @@
         <v>93.19</v>
       </c>
     </row>
-    <row r="6" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="18" t="str">
         <f>IF(Cadastro!B6="","",Cadastro!B6)</f>
         <v>Energia</v>
@@ -9887,7 +9873,7 @@
         <v>145.19000000000003</v>
       </c>
     </row>
-    <row r="7" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="18" t="str">
         <f>IF(Cadastro!B7="","",Cadastro!B7)</f>
         <v>Seguro galpão</v>
@@ -9937,7 +9923,7 @@
         <v>367.0385714285714</v>
       </c>
     </row>
-    <row r="8" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="18" t="str">
         <f>IF(Cadastro!B8="","",Cadastro!B8)</f>
         <v>Segurança Emive</v>
@@ -9991,7 +9977,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="9" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="18" t="str">
         <f>IF(Cadastro!B9="","",Cadastro!B9)</f>
         <v>Dedetização</v>
@@ -10045,7 +10031,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="10" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="18" t="str">
         <f>IF(Cadastro!B10="","",Cadastro!B10)</f>
         <v>IPTU</v>
@@ -10099,7 +10085,7 @@
         <v>321.15875</v>
       </c>
     </row>
-    <row r="11" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="18" t="str">
         <f>IF(Cadastro!B11="","",Cadastro!B11)</f>
         <v>Controle de Ponto</v>
@@ -10153,7 +10139,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="12" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="18" t="str">
         <f>IF(Cadastro!B12="","",Cadastro!B12)</f>
         <v>Extintores</v>
@@ -10207,7 +10193,7 @@
         <v>71.25</v>
       </c>
     </row>
-    <row r="13" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="18" t="str">
         <f>IF(Cadastro!B13="","",Cadastro!B13)</f>
         <v>Internet</v>
@@ -10261,7 +10247,7 @@
         <v>167.71</v>
       </c>
     </row>
-    <row r="14" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="18" t="str">
         <f>IF(Cadastro!B14="","",Cadastro!B14)</f>
         <v>Funcionários</v>
@@ -10315,7 +10301,7 @@
         <v>14212.81</v>
       </c>
     </row>
-    <row r="15" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="18" t="s">
         <v>101</v>
       </c>
@@ -10363,7 +10349,7 @@
         <v>3841.6275000000001</v>
       </c>
     </row>
-    <row r="16" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="55" t="s">
         <v>110</v>
       </c>
@@ -10398,7 +10384,7 @@
         <v>3177.6666666666665</v>
       </c>
     </row>
-    <row r="17" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="18" t="str">
         <f>IF(Cadastro!B17="","",Cadastro!B17)</f>
         <v>Tubete</v>
@@ -10444,7 +10430,7 @@
         <v>14035.15</v>
       </c>
     </row>
-    <row r="18" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="18" t="str">
         <f>IF(Cadastro!B18="","",Cadastro!B18)</f>
         <v>Manutenção Predial</v>
@@ -10488,7 +10474,7 @@
         <v>599.71428571428567</v>
       </c>
     </row>
-    <row r="19" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="18" t="str">
         <f>IF(Cadastro!B19="","",Cadastro!B19)</f>
         <v>Seguro do Caminhão</v>
@@ -10534,7 +10520,7 @@
         <v>464.31166666666599</v>
       </c>
     </row>
-    <row r="20" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="55" t="str">
         <f>IF(Cadastro!B20="","",Cadastro!B20)</f>
         <v>Parcela Caminhão</v>
@@ -10580,7 +10566,7 @@
         <v>3379.4899999999989</v>
       </c>
     </row>
-    <row r="21" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="55" t="str">
         <f>IF(Cadastro!B21="","",Cadastro!B21)</f>
         <v>Despesas Pessoal (EPI, Farda e Ferramentas, Diaristas)</v>
@@ -10613,7 +10599,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="22" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="18" t="str">
         <f>IF(Cadastro!B22="","",Cadastro!B22)</f>
         <v xml:space="preserve">Outras Despesas </v>
@@ -10658,7 +10644,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="24" t="s">
         <v>55</v>
       </c>
@@ -10722,7 +10708,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" errorTitle="Valor inválido" error="Digite apenas números (valor em R$)." sqref="C17:N22 K16:N16 C5:N15">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" errorTitle="Valor inválido" error="Digite apenas números (valor em R$)." sqref="C17:N22 K16:N16 C5:N15" xr:uid="{00000000-0002-0000-0300-000000000000}">
       <formula1>0</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -10733,18 +10719,18 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <sheetPr>
     <tabColor rgb="FF70AD47"/>
   </sheetPr>
   <dimension ref="A1:L23"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5" style="1" customWidth="1"/>
-    <col min="2" max="2" width="52.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="52.88671875" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="20" style="1" customWidth="1"/>
     <col min="4" max="5" width="14" style="1" customWidth="1"/>
-    <col min="6" max="6" width="16.7109375" style="1" customWidth="1"/>
+    <col min="6" max="6" width="16.6640625" style="1" customWidth="1"/>
     <col min="7" max="7" width="11" style="1" customWidth="1"/>
     <col min="8" max="9" width="16" style="1" customWidth="1"/>
     <col min="10" max="10" width="34" style="1" customWidth="1"/>
@@ -10752,12 +10738,12 @@
     <col min="12" max="12" width="20" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="13" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="14" t="s">
         <v>67</v>
       </c>
@@ -10768,7 +10754,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="17" t="s">
         <v>69</v>
       </c>
@@ -10803,7 +10789,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="47">
         <v>1</v>
       </c>
@@ -10834,7 +10820,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="47">
         <v>2</v>
       </c>
@@ -10865,7 +10851,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="47">
         <v>3</v>
       </c>
@@ -10900,7 +10886,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="47">
         <v>4</v>
       </c>
@@ -10931,7 +10917,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="47">
         <v>5</v>
       </c>
@@ -10966,7 +10952,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="10" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="47">
         <v>6</v>
       </c>
@@ -11001,7 +10987,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="11" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="47">
         <v>7</v>
       </c>
@@ -11032,7 +11018,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="12" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="47">
         <v>8</v>
       </c>
@@ -11067,7 +11053,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="13" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="47">
         <v>9</v>
       </c>
@@ -11098,7 +11084,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="14" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="47">
         <v>10</v>
       </c>
@@ -11127,7 +11113,7 @@
       <c r="J14" s="50"/>
       <c r="L14" s="48"/>
     </row>
-    <row r="15" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="47">
         <v>14</v>
       </c>
@@ -11151,7 +11137,7 @@
       <c r="I15" s="20"/>
       <c r="J15" s="50"/>
     </row>
-    <row r="16" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="47">
         <v>15</v>
       </c>
@@ -11178,7 +11164,7 @@
       </c>
       <c r="J16" s="50"/>
     </row>
-    <row r="17" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="47">
         <v>16</v>
       </c>
@@ -11205,7 +11191,7 @@
       </c>
       <c r="J17" s="50"/>
     </row>
-    <row r="18" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="47">
         <v>17</v>
       </c>
@@ -11232,7 +11218,7 @@
       </c>
       <c r="J18" s="50"/>
     </row>
-    <row r="19" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="47">
         <v>18</v>
       </c>
@@ -11259,7 +11245,7 @@
       </c>
       <c r="J19" s="50"/>
     </row>
-    <row r="20" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="47">
         <v>19</v>
       </c>
@@ -11286,7 +11272,7 @@
       </c>
       <c r="J20" s="50"/>
     </row>
-    <row r="21" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="47">
         <v>20</v>
       </c>
@@ -11313,7 +11299,7 @@
       </c>
       <c r="J21" s="50"/>
     </row>
-    <row r="22" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="47">
         <v>21</v>
       </c>
@@ -11340,7 +11326,7 @@
       </c>
       <c r="J22" s="50"/>
     </row>
-    <row r="23" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="51"/>
       <c r="B23" s="51" t="s">
         <v>99</v>
@@ -11362,15 +11348,15 @@
     </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" sqref="E5:E22">
+    <dataValidation type="list" allowBlank="1" sqref="E5:E22" xr:uid="{00000000-0002-0000-0400-000000000000}">
       <formula1>"Mensal,Trimestral,Semestral,Anual"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="C5:C22">
+    <dataValidation type="list" allowBlank="1" sqref="C5:C22" xr:uid="{00000000-0002-0000-0400-000001000000}">
       <formula1>OFFSET($L$5,0,0,COUNTA($L$5:$L$28),1)</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation type="whole" allowBlank="1" sqref="F5:F22">
+    <dataValidation type="whole" allowBlank="1" sqref="F5:F22" xr:uid="{00000000-0002-0000-0400-000002000000}">
       <formula1>1</formula1>
       <formula2>12</formula2>
     </dataValidation>

</xml_diff>